<commit_message>
Dados planilha atualizado V3 	modified:   dados/catalogo.xlsx
</commit_message>
<xml_diff>
--- a/dados/catalogo.xlsx
+++ b/dados/catalogo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leool\Downloads\1. Projetos\App_Python\Consultar_imagens\Consulta_estoque\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB51344F-9CA6-45AD-A6D2-E89CEDA69DA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6440BE4-C185-403D-8CA0-1822F416B7FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2659,7 +2659,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2673,6 +2673,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2968,7 +2969,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="9.140625" customWidth="1"/>
-    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" style="5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="20.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3012,7 +3013,7 @@
         <f t="shared" ref="E2:E65" si="0">IF(F2&gt;0,"Estoque","Acabou")</f>
         <v>Acabou</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="5">
         <v>0</v>
       </c>
       <c r="G2">
@@ -3038,7 +3039,7 @@
         <f t="shared" si="0"/>
         <v>Estoque</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="5">
         <v>1</v>
       </c>
       <c r="G3">
@@ -3066,7 +3067,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="5">
         <v>0</v>
       </c>
       <c r="G4">
@@ -3094,7 +3095,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="5">
         <v>0</v>
       </c>
       <c r="G5">
@@ -3122,7 +3123,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="5">
         <v>0</v>
       </c>
       <c r="G6">
@@ -3150,7 +3151,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="5">
         <v>0</v>
       </c>
       <c r="G7">
@@ -3178,7 +3179,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="5">
         <v>0</v>
       </c>
       <c r="G8">
@@ -3206,7 +3207,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="5">
         <v>0</v>
       </c>
       <c r="G9">
@@ -3234,7 +3235,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="5">
         <v>0</v>
       </c>
       <c r="G10">
@@ -3262,7 +3263,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="5">
         <v>0</v>
       </c>
       <c r="G11">
@@ -3290,7 +3291,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="5">
         <v>0</v>
       </c>
       <c r="G12">
@@ -3318,7 +3319,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="5">
         <v>0</v>
       </c>
       <c r="G13">
@@ -3346,7 +3347,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="5">
         <v>0</v>
       </c>
       <c r="G14">
@@ -3374,7 +3375,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="5">
         <v>0</v>
       </c>
       <c r="G15">
@@ -3402,7 +3403,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="5">
         <v>0</v>
       </c>
       <c r="G16">
@@ -3430,7 +3431,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="5">
         <v>0</v>
       </c>
       <c r="G17">
@@ -3458,7 +3459,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="5">
         <v>0</v>
       </c>
       <c r="G18">
@@ -3486,7 +3487,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="5">
         <v>0</v>
       </c>
       <c r="G19">
@@ -3514,7 +3515,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="5">
         <v>0</v>
       </c>
       <c r="G20">
@@ -3542,7 +3543,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="5">
         <v>0</v>
       </c>
       <c r="G21">
@@ -3570,7 +3571,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="5">
         <v>0</v>
       </c>
       <c r="G22">
@@ -3598,7 +3599,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="5">
         <v>0</v>
       </c>
       <c r="G23">
@@ -3626,7 +3627,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="5">
         <v>0</v>
       </c>
       <c r="G24">
@@ -3654,7 +3655,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="5">
         <v>0</v>
       </c>
       <c r="G25">
@@ -3682,7 +3683,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="5">
         <v>0</v>
       </c>
       <c r="G26">
@@ -3710,7 +3711,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="5">
         <v>0</v>
       </c>
       <c r="G27">
@@ -3738,7 +3739,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F28">
+      <c r="F28" s="5">
         <v>0</v>
       </c>
       <c r="G28">
@@ -3766,7 +3767,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F29">
+      <c r="F29" s="5">
         <v>0</v>
       </c>
       <c r="G29">
@@ -3794,7 +3795,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="5">
         <v>0</v>
       </c>
       <c r="G30">
@@ -3822,7 +3823,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F31">
+      <c r="F31" s="5">
         <v>0</v>
       </c>
       <c r="G31">
@@ -3850,7 +3851,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F32">
+      <c r="F32" s="5">
         <v>0</v>
       </c>
       <c r="G32">
@@ -3878,7 +3879,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="5">
         <v>0</v>
       </c>
       <c r="G33">
@@ -3906,7 +3907,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F34">
+      <c r="F34" s="5">
         <v>0</v>
       </c>
       <c r="G34">
@@ -3934,7 +3935,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F35">
+      <c r="F35" s="5">
         <v>0</v>
       </c>
       <c r="G35">
@@ -3962,7 +3963,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F36">
+      <c r="F36" s="5">
         <v>0</v>
       </c>
       <c r="G36">
@@ -3990,7 +3991,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="5">
         <v>0</v>
       </c>
       <c r="G37">
@@ -4018,7 +4019,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F38">
+      <c r="F38" s="5">
         <v>0</v>
       </c>
       <c r="G38">
@@ -4046,7 +4047,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="5">
         <v>0</v>
       </c>
       <c r="G39">
@@ -4074,7 +4075,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F40">
+      <c r="F40" s="5">
         <v>0</v>
       </c>
       <c r="G40">
@@ -4102,7 +4103,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F41">
+      <c r="F41" s="5">
         <v>0</v>
       </c>
       <c r="G41">
@@ -4130,7 +4131,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F42">
+      <c r="F42" s="5">
         <v>0</v>
       </c>
       <c r="G42">
@@ -4158,7 +4159,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F43">
+      <c r="F43" s="5">
         <v>0</v>
       </c>
       <c r="G43">
@@ -4186,7 +4187,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F44">
+      <c r="F44" s="5">
         <v>0</v>
       </c>
       <c r="G44">
@@ -4214,7 +4215,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F45">
+      <c r="F45" s="5">
         <v>0</v>
       </c>
       <c r="G45">
@@ -4242,7 +4243,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F46">
+      <c r="F46" s="5">
         <v>0</v>
       </c>
       <c r="G46">
@@ -4270,7 +4271,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F47">
+      <c r="F47" s="5">
         <v>0</v>
       </c>
       <c r="G47">
@@ -4298,7 +4299,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F48">
+      <c r="F48" s="5">
         <v>0</v>
       </c>
       <c r="G48">
@@ -4326,7 +4327,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F49">
+      <c r="F49" s="5">
         <v>0</v>
       </c>
       <c r="G49">
@@ -4354,7 +4355,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F50">
+      <c r="F50" s="5">
         <v>0</v>
       </c>
       <c r="G50">
@@ -4382,7 +4383,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F51">
+      <c r="F51" s="5">
         <v>0</v>
       </c>
       <c r="G51">
@@ -4410,7 +4411,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F52">
+      <c r="F52" s="5">
         <v>0</v>
       </c>
       <c r="G52">
@@ -4438,7 +4439,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F53">
+      <c r="F53" s="5">
         <v>0</v>
       </c>
       <c r="G53">
@@ -4466,7 +4467,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F54">
+      <c r="F54" s="5">
         <v>0</v>
       </c>
       <c r="G54">
@@ -4494,7 +4495,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F55">
+      <c r="F55" s="5">
         <v>0</v>
       </c>
       <c r="G55">
@@ -4522,7 +4523,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F56">
+      <c r="F56" s="5">
         <v>0</v>
       </c>
       <c r="G56">
@@ -4550,7 +4551,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F57">
+      <c r="F57" s="5">
         <v>0</v>
       </c>
       <c r="G57">
@@ -4578,7 +4579,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F58">
+      <c r="F58" s="5">
         <v>0</v>
       </c>
       <c r="G58">
@@ -4606,7 +4607,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F59">
+      <c r="F59" s="5">
         <v>0</v>
       </c>
       <c r="G59">
@@ -4634,7 +4635,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F60">
+      <c r="F60" s="5">
         <v>0</v>
       </c>
       <c r="G60">
@@ -4662,7 +4663,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F61">
+      <c r="F61" s="5">
         <v>0</v>
       </c>
       <c r="G61">
@@ -4690,7 +4691,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F62">
+      <c r="F62" s="5">
         <v>0</v>
       </c>
       <c r="G62">
@@ -4718,7 +4719,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F63">
+      <c r="F63" s="5">
         <v>0</v>
       </c>
       <c r="G63">
@@ -4746,7 +4747,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F64">
+      <c r="F64" s="5">
         <v>0</v>
       </c>
       <c r="G64">
@@ -4774,7 +4775,7 @@
         <f t="shared" si="0"/>
         <v>Acabou</v>
       </c>
-      <c r="F65">
+      <c r="F65" s="5">
         <v>0</v>
       </c>
       <c r="G65">
@@ -4802,7 +4803,7 @@
         <f t="shared" ref="E66:E129" si="1">IF(F66&gt;0,"Estoque","Acabou")</f>
         <v>Acabou</v>
       </c>
-      <c r="F66">
+      <c r="F66" s="5">
         <v>0</v>
       </c>
       <c r="G66">
@@ -4830,7 +4831,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F67">
+      <c r="F67" s="5">
         <v>0</v>
       </c>
       <c r="G67">
@@ -4858,7 +4859,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F68">
+      <c r="F68" s="5">
         <v>0</v>
       </c>
       <c r="G68">
@@ -4886,7 +4887,7 @@
         <f t="shared" si="1"/>
         <v>Estoque</v>
       </c>
-      <c r="F69">
+      <c r="F69" s="5">
         <v>1</v>
       </c>
       <c r="G69">
@@ -4914,7 +4915,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F70">
+      <c r="F70" s="5">
         <v>0</v>
       </c>
       <c r="G70">
@@ -4942,7 +4943,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F71">
+      <c r="F71" s="5">
         <v>0</v>
       </c>
       <c r="G71">
@@ -4970,7 +4971,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F72">
+      <c r="F72" s="5">
         <v>0</v>
       </c>
       <c r="G72">
@@ -4998,7 +4999,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F73">
+      <c r="F73" s="5">
         <v>0</v>
       </c>
       <c r="G73">
@@ -5026,7 +5027,7 @@
         <f t="shared" si="1"/>
         <v>Estoque</v>
       </c>
-      <c r="F74">
+      <c r="F74" s="5">
         <v>1</v>
       </c>
       <c r="G74">
@@ -5054,7 +5055,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F75">
+      <c r="F75" s="5">
         <v>0</v>
       </c>
       <c r="G75">
@@ -5082,7 +5083,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F76">
+      <c r="F76" s="5">
         <v>0</v>
       </c>
       <c r="G76">
@@ -5110,7 +5111,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F77">
+      <c r="F77" s="5">
         <v>0</v>
       </c>
       <c r="G77">
@@ -5138,7 +5139,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F78">
+      <c r="F78" s="5">
         <v>0</v>
       </c>
       <c r="G78">
@@ -5166,7 +5167,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F79">
+      <c r="F79" s="5">
         <v>0</v>
       </c>
       <c r="G79">
@@ -5194,7 +5195,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F80">
+      <c r="F80" s="5">
         <v>0</v>
       </c>
       <c r="G80">
@@ -5222,7 +5223,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F81">
+      <c r="F81" s="5">
         <v>0</v>
       </c>
       <c r="G81">
@@ -5250,7 +5251,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F82">
+      <c r="F82" s="5">
         <v>0</v>
       </c>
       <c r="G82">
@@ -5278,7 +5279,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F83">
+      <c r="F83" s="5">
         <v>0</v>
       </c>
       <c r="G83">
@@ -5306,7 +5307,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F84">
+      <c r="F84" s="5">
         <v>0</v>
       </c>
       <c r="G84">
@@ -5334,7 +5335,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F85">
+      <c r="F85" s="5">
         <v>0</v>
       </c>
       <c r="G85">
@@ -5362,7 +5363,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F86">
+      <c r="F86" s="5">
         <v>0</v>
       </c>
       <c r="G86">
@@ -5390,7 +5391,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F87">
+      <c r="F87" s="5">
         <v>0</v>
       </c>
       <c r="G87">
@@ -5418,7 +5419,7 @@
         <f t="shared" si="1"/>
         <v>Estoque</v>
       </c>
-      <c r="F88">
+      <c r="F88" s="5">
         <v>1</v>
       </c>
       <c r="G88">
@@ -5446,7 +5447,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F89">
+      <c r="F89" s="5">
         <v>0</v>
       </c>
       <c r="G89">
@@ -5474,7 +5475,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F90">
+      <c r="F90" s="5">
         <v>0</v>
       </c>
       <c r="G90">
@@ -5502,7 +5503,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F91">
+      <c r="F91" s="5">
         <v>0</v>
       </c>
       <c r="G91">
@@ -5530,7 +5531,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F92">
+      <c r="F92" s="5">
         <v>0</v>
       </c>
       <c r="G92">
@@ -5558,7 +5559,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F93">
+      <c r="F93" s="5">
         <v>0</v>
       </c>
       <c r="G93">
@@ -5586,7 +5587,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F94">
+      <c r="F94" s="5">
         <v>0</v>
       </c>
       <c r="G94">
@@ -5614,7 +5615,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F95">
+      <c r="F95" s="5">
         <v>0</v>
       </c>
       <c r="G95">
@@ -5642,7 +5643,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F96">
+      <c r="F96" s="5">
         <v>0</v>
       </c>
       <c r="G96">
@@ -5670,7 +5671,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F97">
+      <c r="F97" s="5">
         <v>0</v>
       </c>
       <c r="G97">
@@ -5698,7 +5699,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F98">
+      <c r="F98" s="5">
         <v>0</v>
       </c>
       <c r="G98">
@@ -5726,7 +5727,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F99">
+      <c r="F99" s="5">
         <v>0</v>
       </c>
       <c r="G99">
@@ -5754,7 +5755,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F100">
+      <c r="F100" s="5">
         <v>0</v>
       </c>
       <c r="G100">
@@ -5782,7 +5783,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F101">
+      <c r="F101" s="5">
         <v>0</v>
       </c>
       <c r="G101">
@@ -5810,7 +5811,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F102">
+      <c r="F102" s="5">
         <v>0</v>
       </c>
       <c r="G102">
@@ -5838,7 +5839,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F103">
+      <c r="F103" s="5">
         <v>0</v>
       </c>
       <c r="G103">
@@ -5866,7 +5867,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F104">
+      <c r="F104" s="5">
         <v>0</v>
       </c>
       <c r="G104">
@@ -5894,7 +5895,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F105">
+      <c r="F105" s="5">
         <v>0</v>
       </c>
       <c r="G105">
@@ -5922,7 +5923,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F106">
+      <c r="F106" s="5">
         <v>0</v>
       </c>
       <c r="G106">
@@ -5950,7 +5951,7 @@
         <f t="shared" si="1"/>
         <v>Estoque</v>
       </c>
-      <c r="F107">
+      <c r="F107" s="5">
         <v>1</v>
       </c>
       <c r="G107">
@@ -5978,7 +5979,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F108">
+      <c r="F108" s="5">
         <v>0</v>
       </c>
       <c r="G108">
@@ -6006,7 +6007,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F109">
+      <c r="F109" s="5">
         <v>0</v>
       </c>
       <c r="G109">
@@ -6034,7 +6035,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F110">
+      <c r="F110" s="5">
         <v>0</v>
       </c>
       <c r="G110">
@@ -6062,7 +6063,7 @@
         <f t="shared" si="1"/>
         <v>Estoque</v>
       </c>
-      <c r="F111">
+      <c r="F111" s="5">
         <v>1</v>
       </c>
       <c r="G111">
@@ -6090,7 +6091,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F112">
+      <c r="F112" s="5">
         <v>0</v>
       </c>
       <c r="G112">
@@ -6118,7 +6119,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F113">
+      <c r="F113" s="5">
         <v>0</v>
       </c>
       <c r="G113">
@@ -6146,7 +6147,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F114">
+      <c r="F114" s="5">
         <v>0</v>
       </c>
       <c r="G114">
@@ -6174,7 +6175,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F115">
+      <c r="F115" s="5">
         <v>0</v>
       </c>
       <c r="G115">
@@ -6202,7 +6203,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F116">
+      <c r="F116" s="5">
         <v>0</v>
       </c>
       <c r="G116">
@@ -6230,7 +6231,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F117">
+      <c r="F117" s="5">
         <v>0</v>
       </c>
       <c r="G117">
@@ -6258,7 +6259,7 @@
         <f t="shared" si="1"/>
         <v>Estoque</v>
       </c>
-      <c r="F118">
+      <c r="F118" s="5">
         <v>1</v>
       </c>
       <c r="G118">
@@ -6286,7 +6287,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F119">
+      <c r="F119" s="5">
         <v>0</v>
       </c>
       <c r="G119">
@@ -6314,7 +6315,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F120">
+      <c r="F120" s="5">
         <v>0</v>
       </c>
       <c r="G120">
@@ -6342,7 +6343,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F121">
+      <c r="F121" s="5">
         <v>0</v>
       </c>
       <c r="G121">
@@ -6370,7 +6371,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F122">
+      <c r="F122" s="5">
         <v>0</v>
       </c>
       <c r="G122">
@@ -6398,7 +6399,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F123">
+      <c r="F123" s="5">
         <v>0</v>
       </c>
       <c r="G123">
@@ -6426,7 +6427,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F124">
+      <c r="F124" s="5">
         <v>0</v>
       </c>
       <c r="G124">
@@ -6454,7 +6455,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F125">
+      <c r="F125" s="5">
         <v>0</v>
       </c>
       <c r="G125">
@@ -6482,7 +6483,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F126">
+      <c r="F126" s="5">
         <v>0</v>
       </c>
       <c r="G126">
@@ -6510,7 +6511,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F127">
+      <c r="F127" s="5">
         <v>0</v>
       </c>
       <c r="G127">
@@ -6538,7 +6539,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F128">
+      <c r="F128" s="5">
         <v>0</v>
       </c>
       <c r="G128">
@@ -6566,7 +6567,7 @@
         <f t="shared" si="1"/>
         <v>Acabou</v>
       </c>
-      <c r="F129">
+      <c r="F129" s="5">
         <v>0</v>
       </c>
       <c r="G129">
@@ -6594,7 +6595,7 @@
         <f t="shared" ref="E130:E193" si="2">IF(F130&gt;0,"Estoque","Acabou")</f>
         <v>Acabou</v>
       </c>
-      <c r="F130">
+      <c r="F130" s="5">
         <v>0</v>
       </c>
       <c r="G130">
@@ -6622,7 +6623,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F131">
+      <c r="F131" s="5">
         <v>0</v>
       </c>
       <c r="G131">
@@ -6650,7 +6651,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F132">
+      <c r="F132" s="5">
         <v>0</v>
       </c>
       <c r="G132">
@@ -6678,7 +6679,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F133">
+      <c r="F133" s="5">
         <v>0</v>
       </c>
       <c r="G133">
@@ -6706,7 +6707,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F134">
+      <c r="F134" s="5">
         <v>0</v>
       </c>
       <c r="G134">
@@ -6734,7 +6735,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F135">
+      <c r="F135" s="5">
         <v>0</v>
       </c>
       <c r="G135">
@@ -6762,7 +6763,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F136">
+      <c r="F136" s="5">
         <v>0</v>
       </c>
       <c r="G136">
@@ -6790,7 +6791,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F137">
+      <c r="F137" s="5">
         <v>0</v>
       </c>
       <c r="G137">
@@ -6818,7 +6819,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F138">
+      <c r="F138" s="5">
         <v>0</v>
       </c>
       <c r="G138">
@@ -6846,7 +6847,7 @@
         <f t="shared" si="2"/>
         <v>Estoque</v>
       </c>
-      <c r="F139">
+      <c r="F139" s="5">
         <v>1</v>
       </c>
       <c r="G139">
@@ -6874,7 +6875,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F140">
+      <c r="F140" s="5">
         <v>0</v>
       </c>
       <c r="G140">
@@ -6902,7 +6903,7 @@
         <f t="shared" si="2"/>
         <v>Estoque</v>
       </c>
-      <c r="F141">
+      <c r="F141" s="5">
         <v>2</v>
       </c>
       <c r="G141">
@@ -6930,7 +6931,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F142">
+      <c r="F142" s="5">
         <v>0</v>
       </c>
       <c r="G142">
@@ -6958,7 +6959,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F143">
+      <c r="F143" s="5">
         <v>0</v>
       </c>
       <c r="G143">
@@ -6986,7 +6987,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F144">
+      <c r="F144" s="5">
         <v>0</v>
       </c>
       <c r="G144">
@@ -7014,7 +7015,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F145">
+      <c r="F145" s="5">
         <v>0</v>
       </c>
       <c r="G145">
@@ -7042,7 +7043,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F146">
+      <c r="F146" s="5">
         <v>0</v>
       </c>
       <c r="G146">
@@ -7070,7 +7071,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F147">
+      <c r="F147" s="5">
         <v>0</v>
       </c>
       <c r="G147">
@@ -7098,7 +7099,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F148">
+      <c r="F148" s="5">
         <v>0</v>
       </c>
       <c r="G148">
@@ -7126,7 +7127,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F149">
+      <c r="F149" s="5">
         <v>0</v>
       </c>
       <c r="G149">
@@ -7154,7 +7155,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F150">
+      <c r="F150" s="5">
         <v>0</v>
       </c>
       <c r="G150">
@@ -7182,7 +7183,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F151">
+      <c r="F151" s="5">
         <v>0</v>
       </c>
       <c r="G151">
@@ -7210,7 +7211,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F152">
+      <c r="F152" s="5">
         <v>0</v>
       </c>
       <c r="G152">
@@ -7238,7 +7239,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F153">
+      <c r="F153" s="5">
         <v>0</v>
       </c>
       <c r="G153">
@@ -7266,7 +7267,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F154">
+      <c r="F154" s="5">
         <v>0</v>
       </c>
       <c r="G154">
@@ -7294,7 +7295,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F155">
+      <c r="F155" s="5">
         <v>0</v>
       </c>
       <c r="G155">
@@ -7322,7 +7323,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F156">
+      <c r="F156" s="5">
         <v>0</v>
       </c>
       <c r="G156">
@@ -7350,7 +7351,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F157">
+      <c r="F157" s="5">
         <v>0</v>
       </c>
       <c r="G157">
@@ -7378,7 +7379,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F158">
+      <c r="F158" s="5">
         <v>0</v>
       </c>
       <c r="G158">
@@ -7406,7 +7407,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F159">
+      <c r="F159" s="5">
         <v>0</v>
       </c>
       <c r="G159">
@@ -7434,7 +7435,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F160">
+      <c r="F160" s="5">
         <v>0</v>
       </c>
       <c r="G160">
@@ -7462,7 +7463,7 @@
         <f t="shared" si="2"/>
         <v>Estoque</v>
       </c>
-      <c r="F161">
+      <c r="F161" s="5">
         <v>1</v>
       </c>
       <c r="G161">
@@ -7490,7 +7491,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F162">
+      <c r="F162" s="5">
         <v>0</v>
       </c>
       <c r="G162">
@@ -7518,7 +7519,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F163">
+      <c r="F163" s="5">
         <v>0</v>
       </c>
       <c r="G163">
@@ -7546,7 +7547,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F164">
+      <c r="F164" s="5">
         <v>0</v>
       </c>
       <c r="G164">
@@ -7574,7 +7575,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F165">
+      <c r="F165" s="5">
         <v>0</v>
       </c>
       <c r="G165">
@@ -7602,7 +7603,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F166">
+      <c r="F166" s="5">
         <v>0</v>
       </c>
       <c r="G166">
@@ -7630,7 +7631,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F167">
+      <c r="F167" s="5">
         <v>0</v>
       </c>
       <c r="G167">
@@ -7658,7 +7659,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F168">
+      <c r="F168" s="5">
         <v>0</v>
       </c>
       <c r="G168">
@@ -7686,7 +7687,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F169">
+      <c r="F169" s="5">
         <v>0</v>
       </c>
       <c r="G169">
@@ -7714,7 +7715,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F170">
+      <c r="F170" s="5">
         <v>0</v>
       </c>
       <c r="G170">
@@ -7742,7 +7743,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F171">
+      <c r="F171" s="5">
         <v>0</v>
       </c>
       <c r="G171">
@@ -7770,7 +7771,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F172">
+      <c r="F172" s="5">
         <v>0</v>
       </c>
       <c r="G172">
@@ -7798,7 +7799,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F173">
+      <c r="F173" s="5">
         <v>0</v>
       </c>
       <c r="G173">
@@ -7826,7 +7827,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F174">
+      <c r="F174" s="5">
         <v>0</v>
       </c>
       <c r="G174">
@@ -7854,7 +7855,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F175">
+      <c r="F175" s="5">
         <v>0</v>
       </c>
       <c r="G175">
@@ -7882,7 +7883,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F176">
+      <c r="F176" s="5">
         <v>0</v>
       </c>
       <c r="G176">
@@ -7910,7 +7911,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F177">
+      <c r="F177" s="5">
         <v>0</v>
       </c>
       <c r="G177">
@@ -7938,7 +7939,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F178">
+      <c r="F178" s="5">
         <v>0</v>
       </c>
       <c r="G178">
@@ -7966,7 +7967,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F179">
+      <c r="F179" s="5">
         <v>0</v>
       </c>
       <c r="G179">
@@ -7994,7 +7995,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F180">
+      <c r="F180" s="5">
         <v>0</v>
       </c>
       <c r="G180">
@@ -8022,7 +8023,7 @@
         <f t="shared" si="2"/>
         <v>Estoque</v>
       </c>
-      <c r="F181">
+      <c r="F181" s="5">
         <v>1</v>
       </c>
       <c r="G181">
@@ -8050,7 +8051,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F182">
+      <c r="F182" s="5">
         <v>0</v>
       </c>
       <c r="G182">
@@ -8078,7 +8079,7 @@
         <f t="shared" si="2"/>
         <v>Estoque</v>
       </c>
-      <c r="F183">
+      <c r="F183" s="5">
         <v>1</v>
       </c>
       <c r="G183">
@@ -8106,7 +8107,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F184">
+      <c r="F184" s="5">
         <v>0</v>
       </c>
       <c r="G184">
@@ -8134,7 +8135,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F185">
+      <c r="F185" s="5">
         <v>0</v>
       </c>
       <c r="G185">
@@ -8162,7 +8163,7 @@
         <f t="shared" si="2"/>
         <v>Estoque</v>
       </c>
-      <c r="F186">
+      <c r="F186" s="5">
         <v>2</v>
       </c>
       <c r="G186">
@@ -8190,7 +8191,7 @@
         <f t="shared" si="2"/>
         <v>Estoque</v>
       </c>
-      <c r="F187">
+      <c r="F187" s="5">
         <v>1</v>
       </c>
       <c r="G187">
@@ -8218,7 +8219,7 @@
         <f t="shared" si="2"/>
         <v>Estoque</v>
       </c>
-      <c r="F188">
+      <c r="F188" s="5">
         <v>1</v>
       </c>
       <c r="G188">
@@ -8246,7 +8247,7 @@
         <f t="shared" si="2"/>
         <v>Estoque</v>
       </c>
-      <c r="F189">
+      <c r="F189" s="5">
         <v>2</v>
       </c>
       <c r="G189">
@@ -8274,7 +8275,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F190">
+      <c r="F190" s="5">
         <v>0</v>
       </c>
       <c r="G190">
@@ -8302,7 +8303,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F191">
+      <c r="F191" s="5">
         <v>0</v>
       </c>
       <c r="G191">
@@ -8330,7 +8331,7 @@
         <f t="shared" si="2"/>
         <v>Estoque</v>
       </c>
-      <c r="F192">
+      <c r="F192" s="5">
         <v>1</v>
       </c>
       <c r="G192">
@@ -8358,7 +8359,7 @@
         <f t="shared" si="2"/>
         <v>Acabou</v>
       </c>
-      <c r="F193">
+      <c r="F193" s="5">
         <v>0</v>
       </c>
       <c r="G193">
@@ -8386,7 +8387,7 @@
         <f t="shared" ref="E194:E257" si="3">IF(F194&gt;0,"Estoque","Acabou")</f>
         <v>Estoque</v>
       </c>
-      <c r="F194">
+      <c r="F194" s="5">
         <v>2</v>
       </c>
       <c r="G194">
@@ -8414,7 +8415,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F195">
+      <c r="F195" s="5">
         <v>0</v>
       </c>
       <c r="G195">
@@ -8442,7 +8443,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F196">
+      <c r="F196" s="5">
         <v>0</v>
       </c>
       <c r="G196">
@@ -8470,7 +8471,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F197">
+      <c r="F197" s="5">
         <v>0</v>
       </c>
       <c r="G197">
@@ -8498,7 +8499,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F198">
+      <c r="F198" s="5">
         <v>0</v>
       </c>
       <c r="G198">
@@ -8526,7 +8527,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F199">
+      <c r="F199" s="5">
         <v>0</v>
       </c>
       <c r="G199">
@@ -8554,7 +8555,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F200">
+      <c r="F200" s="5">
         <v>0</v>
       </c>
       <c r="G200">
@@ -8582,7 +8583,7 @@
         <f t="shared" si="3"/>
         <v>Estoque</v>
       </c>
-      <c r="F201">
+      <c r="F201" s="5">
         <v>2</v>
       </c>
       <c r="G201">
@@ -8610,7 +8611,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F202">
+      <c r="F202" s="5">
         <v>0</v>
       </c>
       <c r="G202">
@@ -8638,7 +8639,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F203">
+      <c r="F203" s="5">
         <v>0</v>
       </c>
       <c r="G203">
@@ -8666,7 +8667,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F204">
+      <c r="F204" s="5">
         <v>0</v>
       </c>
       <c r="G204">
@@ -8694,7 +8695,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F205">
+      <c r="F205" s="5">
         <v>0</v>
       </c>
       <c r="G205">
@@ -8722,7 +8723,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F206">
+      <c r="F206" s="5">
         <v>0</v>
       </c>
       <c r="G206">
@@ -8750,7 +8751,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F207">
+      <c r="F207" s="5">
         <v>0</v>
       </c>
       <c r="G207">
@@ -8778,7 +8779,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F208">
+      <c r="F208" s="5">
         <v>0</v>
       </c>
       <c r="G208">
@@ -8806,7 +8807,7 @@
         <f t="shared" si="3"/>
         <v>Estoque</v>
       </c>
-      <c r="F209">
+      <c r="F209" s="5">
         <v>1</v>
       </c>
       <c r="G209">
@@ -8834,7 +8835,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F210">
+      <c r="F210" s="5">
         <v>0</v>
       </c>
       <c r="G210">
@@ -8862,7 +8863,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F211">
+      <c r="F211" s="5">
         <v>0</v>
       </c>
       <c r="G211">
@@ -8890,7 +8891,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F212">
+      <c r="F212" s="5">
         <v>0</v>
       </c>
       <c r="G212">
@@ -8918,7 +8919,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F213">
+      <c r="F213" s="5">
         <v>0</v>
       </c>
       <c r="G213">
@@ -8946,7 +8947,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F214">
+      <c r="F214" s="5">
         <v>0</v>
       </c>
       <c r="G214">
@@ -8974,7 +8975,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F215">
+      <c r="F215" s="5">
         <v>0</v>
       </c>
       <c r="G215">
@@ -9002,7 +9003,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F216">
+      <c r="F216" s="5">
         <v>0</v>
       </c>
       <c r="G216">
@@ -9030,7 +9031,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F217">
+      <c r="F217" s="5">
         <v>0</v>
       </c>
       <c r="G217">
@@ -9058,7 +9059,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F218">
+      <c r="F218" s="5">
         <v>0</v>
       </c>
       <c r="G218">
@@ -9086,7 +9087,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F219">
+      <c r="F219" s="5">
         <v>0</v>
       </c>
       <c r="G219">
@@ -9114,7 +9115,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F220">
+      <c r="F220" s="5">
         <v>0</v>
       </c>
       <c r="G220">
@@ -9142,7 +9143,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F221">
+      <c r="F221" s="5">
         <v>0</v>
       </c>
       <c r="G221">
@@ -9170,7 +9171,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F222">
+      <c r="F222" s="5">
         <v>0</v>
       </c>
       <c r="G222">
@@ -9198,7 +9199,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F223">
+      <c r="F223" s="5">
         <v>0</v>
       </c>
       <c r="G223">
@@ -9226,7 +9227,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F224">
+      <c r="F224" s="5">
         <v>0</v>
       </c>
       <c r="G224">
@@ -9254,7 +9255,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F225">
+      <c r="F225" s="5">
         <v>0</v>
       </c>
       <c r="G225">
@@ -9282,7 +9283,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F226">
+      <c r="F226" s="5">
         <v>0</v>
       </c>
       <c r="G226">
@@ -9310,7 +9311,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F227">
+      <c r="F227" s="5">
         <v>0</v>
       </c>
       <c r="G227">
@@ -9338,7 +9339,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F228">
+      <c r="F228" s="5">
         <v>0</v>
       </c>
       <c r="G228">
@@ -9366,7 +9367,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F229">
+      <c r="F229" s="5">
         <v>0</v>
       </c>
       <c r="G229">
@@ -9394,7 +9395,7 @@
         <f t="shared" si="3"/>
         <v>Estoque</v>
       </c>
-      <c r="F230">
+      <c r="F230" s="5">
         <v>1</v>
       </c>
       <c r="G230">
@@ -9422,7 +9423,7 @@
         <f t="shared" si="3"/>
         <v>Estoque</v>
       </c>
-      <c r="F231">
+      <c r="F231" s="5">
         <v>1</v>
       </c>
       <c r="G231">
@@ -9450,7 +9451,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F232">
+      <c r="F232" s="5">
         <v>0</v>
       </c>
       <c r="G232">
@@ -9478,7 +9479,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F233">
+      <c r="F233" s="5">
         <v>0</v>
       </c>
       <c r="G233">
@@ -9506,7 +9507,7 @@
         <f t="shared" si="3"/>
         <v>Estoque</v>
       </c>
-      <c r="F234">
+      <c r="F234" s="5">
         <v>1</v>
       </c>
       <c r="G234">
@@ -9534,7 +9535,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F235">
+      <c r="F235" s="5">
         <v>0</v>
       </c>
       <c r="G235">
@@ -9562,7 +9563,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F236">
+      <c r="F236" s="5">
         <v>0</v>
       </c>
       <c r="G236">
@@ -9590,7 +9591,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F237">
+      <c r="F237" s="5">
         <v>0</v>
       </c>
       <c r="G237">
@@ -9618,7 +9619,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F238">
+      <c r="F238" s="5">
         <v>0</v>
       </c>
       <c r="G238">
@@ -9646,7 +9647,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F239">
+      <c r="F239" s="5">
         <v>0</v>
       </c>
       <c r="G239">
@@ -9674,7 +9675,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F240">
+      <c r="F240" s="5">
         <v>0</v>
       </c>
       <c r="G240">
@@ -9702,7 +9703,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F241">
+      <c r="F241" s="5">
         <v>0</v>
       </c>
       <c r="G241">
@@ -9730,7 +9731,7 @@
         <f t="shared" si="3"/>
         <v>Estoque</v>
       </c>
-      <c r="F242">
+      <c r="F242" s="5">
         <v>1</v>
       </c>
       <c r="G242">
@@ -9758,7 +9759,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F243">
+      <c r="F243" s="5">
         <v>0</v>
       </c>
       <c r="G243">
@@ -9786,7 +9787,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F244">
+      <c r="F244" s="5">
         <v>0</v>
       </c>
       <c r="G244">
@@ -9814,7 +9815,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F245">
+      <c r="F245" s="5">
         <v>0</v>
       </c>
       <c r="G245">
@@ -9842,7 +9843,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F246">
+      <c r="F246" s="5">
         <v>0</v>
       </c>
       <c r="G246">
@@ -9870,7 +9871,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F247">
+      <c r="F247" s="5">
         <v>0</v>
       </c>
       <c r="G247">
@@ -9898,7 +9899,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F248">
+      <c r="F248" s="5">
         <v>0</v>
       </c>
       <c r="G248">
@@ -9926,7 +9927,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F249">
+      <c r="F249" s="5">
         <v>0</v>
       </c>
       <c r="G249">
@@ -9954,7 +9955,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F250">
+      <c r="F250" s="5">
         <v>0</v>
       </c>
       <c r="G250">
@@ -9982,7 +9983,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F251">
+      <c r="F251" s="5">
         <v>0</v>
       </c>
       <c r="G251">
@@ -10010,7 +10011,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F252">
+      <c r="F252" s="5">
         <v>0</v>
       </c>
       <c r="G252">
@@ -10038,7 +10039,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F253">
+      <c r="F253" s="5">
         <v>0</v>
       </c>
       <c r="G253">
@@ -10066,7 +10067,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F254">
+      <c r="F254" s="5">
         <v>0</v>
       </c>
       <c r="G254">
@@ -10094,7 +10095,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F255">
+      <c r="F255" s="5">
         <v>0</v>
       </c>
       <c r="G255">
@@ -10122,7 +10123,7 @@
         <f t="shared" si="3"/>
         <v>Acabou</v>
       </c>
-      <c r="F256">
+      <c r="F256" s="5">
         <v>0</v>
       </c>
       <c r="G256">
@@ -10150,7 +10151,7 @@
         <f t="shared" si="3"/>
         <v>Estoque</v>
       </c>
-      <c r="F257">
+      <c r="F257" s="5">
         <v>1</v>
       </c>
       <c r="G257">
@@ -10178,7 +10179,7 @@
         <f t="shared" ref="E258:E321" si="4">IF(F258&gt;0,"Estoque","Acabou")</f>
         <v>Estoque</v>
       </c>
-      <c r="F258">
+      <c r="F258" s="5">
         <v>1</v>
       </c>
       <c r="G258">
@@ -10206,7 +10207,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F259">
+      <c r="F259" s="5">
         <v>0</v>
       </c>
       <c r="G259">
@@ -10234,7 +10235,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F260">
+      <c r="F260" s="5">
         <v>0</v>
       </c>
       <c r="G260">
@@ -10262,7 +10263,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F261">
+      <c r="F261" s="5">
         <v>0</v>
       </c>
       <c r="G261">
@@ -10290,7 +10291,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F262">
+      <c r="F262" s="5">
         <v>0</v>
       </c>
       <c r="G262">
@@ -10318,7 +10319,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F263">
+      <c r="F263" s="5">
         <v>1</v>
       </c>
       <c r="G263">
@@ -10346,7 +10347,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F264">
+      <c r="F264" s="5">
         <v>0</v>
       </c>
       <c r="G264">
@@ -10374,7 +10375,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F265">
+      <c r="F265" s="5">
         <v>1</v>
       </c>
       <c r="G265">
@@ -10402,7 +10403,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F266">
+      <c r="F266" s="5">
         <v>0</v>
       </c>
       <c r="G266">
@@ -10430,7 +10431,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F267">
+      <c r="F267" s="5">
         <v>0</v>
       </c>
       <c r="G267">
@@ -10458,7 +10459,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F268">
+      <c r="F268" s="5">
         <v>0</v>
       </c>
       <c r="G268">
@@ -10486,7 +10487,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F269">
+      <c r="F269" s="5">
         <v>0</v>
       </c>
       <c r="G269">
@@ -10514,7 +10515,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F270">
+      <c r="F270" s="5">
         <v>0</v>
       </c>
       <c r="G270">
@@ -10542,7 +10543,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F271">
+      <c r="F271" s="5">
         <v>0</v>
       </c>
       <c r="G271">
@@ -10570,7 +10571,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F272">
+      <c r="F272" s="5">
         <v>0</v>
       </c>
       <c r="G272">
@@ -10598,7 +10599,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F273">
+      <c r="F273" s="5">
         <v>0</v>
       </c>
       <c r="G273">
@@ -10626,7 +10627,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F274">
+      <c r="F274" s="5">
         <v>1</v>
       </c>
       <c r="G274">
@@ -10654,7 +10655,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F275">
+      <c r="F275" s="5">
         <v>1</v>
       </c>
       <c r="G275">
@@ -10682,7 +10683,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F276">
+      <c r="F276" s="5">
         <v>0</v>
       </c>
       <c r="G276">
@@ -10710,7 +10711,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F277">
+      <c r="F277" s="5">
         <v>2</v>
       </c>
       <c r="G277">
@@ -10738,7 +10739,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F278">
+      <c r="F278" s="5">
         <v>0</v>
       </c>
       <c r="G278">
@@ -10766,7 +10767,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F279">
+      <c r="F279" s="5">
         <v>0</v>
       </c>
       <c r="G279">
@@ -10794,7 +10795,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F280">
+      <c r="F280" s="5">
         <v>0</v>
       </c>
       <c r="G280">
@@ -10822,7 +10823,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F281">
+      <c r="F281" s="5">
         <v>1</v>
       </c>
       <c r="G281">
@@ -10850,7 +10851,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F282">
+      <c r="F282" s="5">
         <v>0</v>
       </c>
       <c r="G282">
@@ -10878,7 +10879,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F283">
+      <c r="F283" s="5">
         <v>0</v>
       </c>
       <c r="G283">
@@ -10906,7 +10907,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F284">
+      <c r="F284" s="5">
         <v>0</v>
       </c>
       <c r="G284">
@@ -10934,7 +10935,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F285">
+      <c r="F285" s="5">
         <v>0</v>
       </c>
       <c r="G285">
@@ -10962,7 +10963,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F286">
+      <c r="F286" s="5">
         <v>0</v>
       </c>
       <c r="G286">
@@ -10990,7 +10991,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F287">
+      <c r="F287" s="5">
         <v>0</v>
       </c>
       <c r="G287">
@@ -11018,7 +11019,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F288">
+      <c r="F288" s="5">
         <v>0</v>
       </c>
       <c r="G288">
@@ -11046,7 +11047,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F289">
+      <c r="F289" s="5">
         <v>1</v>
       </c>
       <c r="G289">
@@ -11074,7 +11075,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F290">
+      <c r="F290" s="5">
         <v>0</v>
       </c>
       <c r="G290">
@@ -11102,7 +11103,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F291">
+      <c r="F291" s="5">
         <v>1</v>
       </c>
       <c r="G291">
@@ -11130,7 +11131,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F292">
+      <c r="F292" s="5">
         <v>2</v>
       </c>
       <c r="G292">
@@ -11158,7 +11159,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F293">
+      <c r="F293" s="5">
         <v>1</v>
       </c>
       <c r="G293">
@@ -11186,7 +11187,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F294">
+      <c r="F294" s="5">
         <v>0</v>
       </c>
       <c r="G294">
@@ -11214,7 +11215,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F295">
+      <c r="F295" s="5">
         <v>1</v>
       </c>
       <c r="G295">
@@ -11242,7 +11243,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F296">
+      <c r="F296" s="5">
         <v>0</v>
       </c>
       <c r="G296">
@@ -11270,7 +11271,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F297">
+      <c r="F297" s="5">
         <v>0</v>
       </c>
       <c r="G297">
@@ -11298,7 +11299,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F298">
+      <c r="F298" s="5">
         <v>0</v>
       </c>
       <c r="G298">
@@ -11326,7 +11327,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F299">
+      <c r="F299" s="5">
         <v>0</v>
       </c>
       <c r="G299">
@@ -11354,7 +11355,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F300">
+      <c r="F300" s="5">
         <v>0</v>
       </c>
       <c r="G300">
@@ -11382,7 +11383,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F301">
+      <c r="F301" s="5">
         <v>1</v>
       </c>
       <c r="G301">
@@ -11410,7 +11411,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F302">
+      <c r="F302" s="5">
         <v>1</v>
       </c>
       <c r="G302">
@@ -11438,7 +11439,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F303">
+      <c r="F303" s="5">
         <v>0</v>
       </c>
       <c r="G303">
@@ -11466,7 +11467,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F304">
+      <c r="F304" s="5">
         <v>0</v>
       </c>
       <c r="G304">
@@ -11494,7 +11495,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F305">
+      <c r="F305" s="5">
         <v>0</v>
       </c>
       <c r="G305">
@@ -11522,7 +11523,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F306">
+      <c r="F306" s="5">
         <v>3</v>
       </c>
       <c r="G306">
@@ -11550,7 +11551,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F307">
+      <c r="F307" s="5">
         <v>1</v>
       </c>
       <c r="G307">
@@ -11578,7 +11579,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F308">
+      <c r="F308" s="5">
         <v>0</v>
       </c>
       <c r="G308">
@@ -11606,7 +11607,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F309">
+      <c r="F309" s="5">
         <v>0</v>
       </c>
       <c r="G309">
@@ -11634,7 +11635,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F310">
+      <c r="F310" s="5">
         <v>0</v>
       </c>
       <c r="G310">
@@ -11662,7 +11663,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F311">
+      <c r="F311" s="5">
         <v>1</v>
       </c>
       <c r="G311">
@@ -11690,7 +11691,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F312">
+      <c r="F312" s="5">
         <v>0</v>
       </c>
       <c r="G312">
@@ -11718,7 +11719,7 @@
         <f t="shared" si="4"/>
         <v>Estoque</v>
       </c>
-      <c r="F313">
+      <c r="F313" s="5">
         <v>1</v>
       </c>
       <c r="G313">
@@ -11746,7 +11747,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F314">
+      <c r="F314" s="5">
         <v>0</v>
       </c>
       <c r="G314">
@@ -11774,7 +11775,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F315">
+      <c r="F315" s="5">
         <v>0</v>
       </c>
       <c r="G315">
@@ -11802,7 +11803,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F316">
+      <c r="F316" s="5">
         <v>0</v>
       </c>
       <c r="G316">
@@ -11830,7 +11831,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F317">
+      <c r="F317" s="5">
         <v>0</v>
       </c>
       <c r="G317">
@@ -11858,7 +11859,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F318">
+      <c r="F318" s="5">
         <v>0</v>
       </c>
       <c r="G318">
@@ -11886,7 +11887,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F319">
+      <c r="F319" s="5">
         <v>0</v>
       </c>
       <c r="G319">
@@ -11914,7 +11915,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F320">
+      <c r="F320" s="5">
         <v>0</v>
       </c>
       <c r="G320">
@@ -11942,7 +11943,7 @@
         <f t="shared" si="4"/>
         <v>Acabou</v>
       </c>
-      <c r="F321">
+      <c r="F321" s="5">
         <v>0</v>
       </c>
       <c r="G321">
@@ -11970,7 +11971,7 @@
         <f t="shared" ref="E322:E384" si="5">IF(F322&gt;0,"Estoque","Acabou")</f>
         <v>Estoque</v>
       </c>
-      <c r="F322">
+      <c r="F322" s="5">
         <v>2</v>
       </c>
       <c r="G322">
@@ -11998,7 +11999,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F323">
+      <c r="F323" s="5">
         <v>0</v>
       </c>
       <c r="G323">
@@ -12026,7 +12027,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F324">
+      <c r="F324" s="5">
         <v>2</v>
       </c>
       <c r="G324">
@@ -12054,7 +12055,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F325">
+      <c r="F325" s="5">
         <v>1</v>
       </c>
       <c r="G325">
@@ -12082,7 +12083,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F326">
+      <c r="F326" s="5">
         <v>1</v>
       </c>
       <c r="G326">
@@ -12110,7 +12111,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F327">
+      <c r="F327" s="5">
         <v>0</v>
       </c>
       <c r="G327">
@@ -12138,7 +12139,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F328">
+      <c r="F328" s="5">
         <v>1</v>
       </c>
       <c r="G328">
@@ -12166,7 +12167,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F329">
+      <c r="F329" s="5">
         <v>0</v>
       </c>
       <c r="G329">
@@ -12194,7 +12195,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F330">
+      <c r="F330" s="5">
         <v>0</v>
       </c>
       <c r="G330">
@@ -12222,7 +12223,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F331">
+      <c r="F331" s="5">
         <v>1</v>
       </c>
       <c r="G331">
@@ -12250,7 +12251,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F332">
+      <c r="F332" s="5">
         <v>0</v>
       </c>
       <c r="G332">
@@ -12278,7 +12279,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F333">
+      <c r="F333" s="5">
         <v>0</v>
       </c>
       <c r="G333">
@@ -12306,7 +12307,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F334">
+      <c r="F334" s="5">
         <v>0</v>
       </c>
       <c r="G334">
@@ -12334,7 +12335,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F335">
+      <c r="F335" s="5">
         <v>0</v>
       </c>
       <c r="G335">
@@ -12362,7 +12363,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F336">
+      <c r="F336" s="5">
         <v>0</v>
       </c>
       <c r="G336">
@@ -12390,7 +12391,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F337">
+      <c r="F337" s="5">
         <v>0</v>
       </c>
       <c r="G337">
@@ -12418,7 +12419,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F338">
+      <c r="F338" s="5">
         <v>0</v>
       </c>
       <c r="G338">
@@ -12446,7 +12447,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F339">
+      <c r="F339" s="5">
         <v>0</v>
       </c>
       <c r="G339">
@@ -12474,7 +12475,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F340">
+      <c r="F340" s="5">
         <v>0</v>
       </c>
       <c r="G340">
@@ -12502,7 +12503,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F341">
+      <c r="F341" s="5">
         <v>0</v>
       </c>
       <c r="G341">
@@ -12530,7 +12531,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F342">
+      <c r="F342" s="5">
         <v>0</v>
       </c>
       <c r="G342">
@@ -12558,7 +12559,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F343">
+      <c r="F343" s="5">
         <v>0</v>
       </c>
       <c r="G343">
@@ -12586,7 +12587,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F344">
+      <c r="F344" s="5">
         <v>0</v>
       </c>
       <c r="G344">
@@ -12614,7 +12615,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F345">
+      <c r="F345" s="5">
         <v>0</v>
       </c>
       <c r="G345">
@@ -12642,7 +12643,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F346">
+      <c r="F346" s="5">
         <v>0</v>
       </c>
       <c r="G346">
@@ -12670,7 +12671,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F347">
+      <c r="F347" s="5">
         <v>0</v>
       </c>
       <c r="G347">
@@ -12698,7 +12699,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F348">
+      <c r="F348" s="5">
         <v>0</v>
       </c>
       <c r="G348">
@@ -12726,7 +12727,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F349">
+      <c r="F349" s="5">
         <v>0</v>
       </c>
       <c r="G349">
@@ -12754,7 +12755,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F350">
+      <c r="F350" s="5">
         <v>3</v>
       </c>
       <c r="G350">
@@ -12782,7 +12783,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F351">
+      <c r="F351" s="5">
         <v>1</v>
       </c>
       <c r="G351">
@@ -12810,7 +12811,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F352">
+      <c r="F352" s="5">
         <v>0</v>
       </c>
       <c r="G352">
@@ -12838,7 +12839,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F353">
+      <c r="F353" s="5">
         <v>1</v>
       </c>
       <c r="G353">
@@ -12866,7 +12867,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F354">
+      <c r="F354" s="5">
         <v>1</v>
       </c>
       <c r="G354">
@@ -12894,7 +12895,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F355">
+      <c r="F355" s="5">
         <v>0</v>
       </c>
       <c r="G355">
@@ -12922,7 +12923,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F356">
+      <c r="F356" s="5">
         <v>0</v>
       </c>
       <c r="G356">
@@ -12950,7 +12951,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F357">
+      <c r="F357" s="5">
         <v>0</v>
       </c>
       <c r="G357">
@@ -12978,7 +12979,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F358">
+      <c r="F358" s="5">
         <v>1</v>
       </c>
       <c r="G358">
@@ -13006,7 +13007,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F359">
+      <c r="F359" s="5">
         <v>0</v>
       </c>
       <c r="G359">
@@ -13034,7 +13035,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F360">
+      <c r="F360" s="5">
         <v>1</v>
       </c>
       <c r="G360">
@@ -13062,7 +13063,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F361">
+      <c r="F361" s="5">
         <v>4</v>
       </c>
       <c r="G361">
@@ -13090,7 +13091,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F362">
+      <c r="F362" s="5">
         <v>0</v>
       </c>
       <c r="G362">
@@ -13118,7 +13119,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F363">
+      <c r="F363" s="5">
         <v>0</v>
       </c>
       <c r="G363">
@@ -13146,7 +13147,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F364">
+      <c r="F364" s="5">
         <v>1</v>
       </c>
       <c r="G364">
@@ -13174,7 +13175,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F365">
+      <c r="F365" s="5">
         <v>0</v>
       </c>
       <c r="G365">
@@ -13202,7 +13203,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F366">
+      <c r="F366" s="5">
         <v>3</v>
       </c>
       <c r="G366">
@@ -13230,7 +13231,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F367">
+      <c r="F367" s="5">
         <v>0</v>
       </c>
       <c r="G367">
@@ -13258,7 +13259,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F368">
+      <c r="F368" s="5">
         <v>1</v>
       </c>
       <c r="G368">
@@ -13286,7 +13287,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F369">
+      <c r="F369" s="5">
         <v>1</v>
       </c>
       <c r="G369">
@@ -13314,7 +13315,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F370">
+      <c r="F370" s="5">
         <v>0</v>
       </c>
       <c r="G370">
@@ -13342,7 +13343,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F371">
+      <c r="F371" s="5">
         <v>1</v>
       </c>
       <c r="G371">
@@ -13370,7 +13371,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F372">
+      <c r="F372" s="5">
         <v>0</v>
       </c>
       <c r="G372">
@@ -13398,7 +13399,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F373">
+      <c r="F373" s="5">
         <v>0</v>
       </c>
       <c r="G373">
@@ -13426,7 +13427,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F374">
+      <c r="F374" s="5">
         <v>2</v>
       </c>
       <c r="G374">
@@ -13454,7 +13455,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F375">
+      <c r="F375" s="5">
         <v>0</v>
       </c>
       <c r="G375">
@@ -13482,7 +13483,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F376">
+      <c r="F376" s="5">
         <v>0</v>
       </c>
       <c r="G376">
@@ -13510,7 +13511,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F377">
+      <c r="F377" s="5">
         <v>0</v>
       </c>
       <c r="G377">
@@ -13538,7 +13539,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F378">
+      <c r="F378" s="5">
         <v>2</v>
       </c>
       <c r="G378">
@@ -13566,7 +13567,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F379">
+      <c r="F379" s="5">
         <v>2</v>
       </c>
       <c r="G379">
@@ -13594,7 +13595,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F380">
+      <c r="F380" s="5">
         <v>2</v>
       </c>
       <c r="G380">
@@ -13622,7 +13623,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F381">
+      <c r="F381" s="5">
         <v>2</v>
       </c>
       <c r="G381">
@@ -13650,7 +13651,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F382">
+      <c r="F382" s="5">
         <v>1</v>
       </c>
       <c r="G382">
@@ -13678,7 +13679,7 @@
         <f t="shared" si="5"/>
         <v>Estoque</v>
       </c>
-      <c r="F383">
+      <c r="F383" s="5">
         <v>1</v>
       </c>
       <c r="G383">
@@ -13706,7 +13707,7 @@
         <f t="shared" si="5"/>
         <v>Acabou</v>
       </c>
-      <c r="F384">
+      <c r="F384" s="5">
         <v>0</v>
       </c>
       <c r="G384">

</xml_diff>

<commit_message>
Dados planilha atualizado V4 	modified:   dados/catalogo.xlsx
</commit_message>
<xml_diff>
--- a/dados/catalogo.xlsx
+++ b/dados/catalogo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leool\Downloads\1. Projetos\App_Python\Consultar_imagens\Consulta_estoque\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6440BE4-C185-403D-8CA0-1822F416B7FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D05AD2CA-F285-4402-B62C-68F036B5B399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1427,9 +1427,6 @@
     <t>qtd</t>
   </si>
   <si>
-    <t>quatidade</t>
-  </si>
-  <si>
     <t>Imagens/#KAL001.jpg</t>
   </si>
   <si>
@@ -2577,6 +2574,9 @@
   </si>
   <si>
     <t>Imagens/Sophis/#SOP016.jpg</t>
+  </si>
+  <si>
+    <t>quantidade</t>
   </si>
 </sst>
 </file>
@@ -2990,7 +2990,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>461</v>
+        <v>844</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>460</v>
@@ -3004,7 +3004,7 @@
         <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D2">
         <v>55</v>
@@ -3030,7 +3030,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="D3">
         <v>30</v>
@@ -3058,7 +3058,7 @@
         <v>9</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="D4">
         <v>36</v>
@@ -3086,7 +3086,7 @@
         <v>10</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="D5">
         <v>36</v>
@@ -3114,7 +3114,7 @@
         <v>12</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="D6">
         <v>35</v>
@@ -3142,7 +3142,7 @@
         <v>13</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="D7">
         <v>55</v>
@@ -3170,7 +3170,7 @@
         <v>15</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="D8">
         <v>60</v>
@@ -3198,7 +3198,7 @@
         <v>16</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="D9">
         <v>80</v>
@@ -3226,7 +3226,7 @@
         <v>17</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D10">
         <v>90</v>
@@ -3254,7 +3254,7 @@
         <v>18</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="D11">
         <v>70</v>
@@ -3282,7 +3282,7 @@
         <v>19</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="D12">
         <v>75</v>
@@ -3310,7 +3310,7 @@
         <v>20</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D13">
         <v>90</v>
@@ -3338,7 +3338,7 @@
         <v>21</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="D14">
         <v>80</v>
@@ -3366,7 +3366,7 @@
         <v>23</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D15">
         <v>35</v>
@@ -3394,7 +3394,7 @@
         <v>24</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="D16">
         <v>85</v>
@@ -3422,7 +3422,7 @@
         <v>25</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="D17">
         <v>70</v>
@@ -3450,7 +3450,7 @@
         <v>26</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="D18">
         <v>85</v>
@@ -3478,7 +3478,7 @@
         <v>28</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="D19">
         <v>55</v>
@@ -3506,7 +3506,7 @@
         <v>29</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="D20">
         <v>55</v>
@@ -3534,7 +3534,7 @@
         <v>30</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="D21">
         <v>55</v>
@@ -3562,7 +3562,7 @@
         <v>31</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="D22">
         <v>55</v>
@@ -3590,7 +3590,7 @@
         <v>32</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="D23">
         <v>55</v>
@@ -3618,7 +3618,7 @@
         <v>33</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="D24">
         <v>50</v>
@@ -3646,7 +3646,7 @@
         <v>34</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="D25">
         <v>50</v>
@@ -3674,7 +3674,7 @@
         <v>35</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="D26">
         <v>55</v>
@@ -3702,7 +3702,7 @@
         <v>36</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D27">
         <v>60</v>
@@ -3730,7 +3730,7 @@
         <v>37</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="D28">
         <v>60</v>
@@ -3758,7 +3758,7 @@
         <v>38</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D29">
         <v>50</v>
@@ -3786,7 +3786,7 @@
         <v>39</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D30">
         <v>50</v>
@@ -3814,7 +3814,7 @@
         <v>40</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="D31">
         <v>55</v>
@@ -3842,7 +3842,7 @@
         <v>41</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="D32">
         <v>60</v>
@@ -3870,7 +3870,7 @@
         <v>42</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="D33">
         <v>55</v>
@@ -3898,7 +3898,7 @@
         <v>43</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="D34">
         <v>55</v>
@@ -3926,7 +3926,7 @@
         <v>44</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="D35">
         <v>50</v>
@@ -3954,7 +3954,7 @@
         <v>45</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="D36">
         <v>50</v>
@@ -3982,7 +3982,7 @@
         <v>46</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="D37">
         <v>55</v>
@@ -4010,7 +4010,7 @@
         <v>47</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="D38">
         <v>55</v>
@@ -4038,7 +4038,7 @@
         <v>48</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D39">
         <v>55</v>
@@ -4066,7 +4066,7 @@
         <v>50</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="D40">
         <v>130</v>
@@ -4094,7 +4094,7 @@
         <v>51</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="D41">
         <v>110</v>
@@ -4122,7 +4122,7 @@
         <v>53</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D42">
         <v>36</v>
@@ -4150,7 +4150,7 @@
         <v>54</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="D43">
         <v>48</v>
@@ -4178,7 +4178,7 @@
         <v>55</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="D44">
         <v>36</v>
@@ -4206,7 +4206,7 @@
         <v>57</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="D45">
         <v>55</v>
@@ -4234,7 +4234,7 @@
         <v>58</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="D46">
         <v>55</v>
@@ -4262,7 +4262,7 @@
         <v>60</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="D47">
         <v>75</v>
@@ -4290,7 +4290,7 @@
         <v>62</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="D48">
         <v>38</v>
@@ -4318,7 +4318,7 @@
         <v>63</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="D49">
         <v>36</v>
@@ -4346,7 +4346,7 @@
         <v>65</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="D50">
         <v>36</v>
@@ -4374,7 +4374,7 @@
         <v>66</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="D51">
         <v>36</v>
@@ -4402,7 +4402,7 @@
         <v>68</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="D52">
         <v>50</v>
@@ -4430,7 +4430,7 @@
         <v>69</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="D53">
         <v>50</v>
@@ -4458,7 +4458,7 @@
         <v>70</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="D54">
         <v>45</v>
@@ -4486,7 +4486,7 @@
         <v>71</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="D55">
         <v>45</v>
@@ -4514,7 +4514,7 @@
         <v>72</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="D56">
         <v>45</v>
@@ -4542,7 +4542,7 @@
         <v>73</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="D57">
         <v>50</v>
@@ -4570,7 +4570,7 @@
         <v>74</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="D58">
         <v>50</v>
@@ -4598,7 +4598,7 @@
         <v>76</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="D59">
         <v>65</v>
@@ -4626,7 +4626,7 @@
         <v>78</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="D60">
         <v>100</v>
@@ -4654,7 +4654,7 @@
         <v>79</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D61">
         <v>110</v>
@@ -4682,7 +4682,7 @@
         <v>80</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="D62">
         <v>115</v>
@@ -4710,7 +4710,7 @@
         <v>81</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="D63">
         <v>150</v>
@@ -4738,7 +4738,7 @@
         <v>82</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="D64">
         <v>115</v>
@@ -4766,7 +4766,7 @@
         <v>83</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="D65">
         <v>150</v>
@@ -4794,7 +4794,7 @@
         <v>84</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="D66">
         <v>150</v>
@@ -4822,7 +4822,7 @@
         <v>86</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="D67">
         <v>55</v>
@@ -4850,7 +4850,7 @@
         <v>87</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="D68">
         <v>55</v>
@@ -4878,7 +4878,7 @@
         <v>88</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D69">
         <v>55</v>
@@ -4906,7 +4906,7 @@
         <v>89</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="D70">
         <v>60</v>
@@ -4934,7 +4934,7 @@
         <v>91</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D71">
         <v>90</v>
@@ -4962,7 +4962,7 @@
         <v>92</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="D72">
         <v>90</v>
@@ -4990,7 +4990,7 @@
         <v>93</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D73">
         <v>80</v>
@@ -5018,7 +5018,7 @@
         <v>95</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="D74">
         <v>130</v>
@@ -5046,7 +5046,7 @@
         <v>96</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="D75">
         <v>130</v>
@@ -5074,7 +5074,7 @@
         <v>98</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="D76">
         <v>65</v>
@@ -5102,7 +5102,7 @@
         <v>99</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="D77">
         <v>60</v>
@@ -5130,7 +5130,7 @@
         <v>100</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="D78">
         <v>60</v>
@@ -5158,7 +5158,7 @@
         <v>101</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="D79">
         <v>60</v>
@@ -5186,7 +5186,7 @@
         <v>102</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="D80">
         <v>60</v>
@@ -5214,7 +5214,7 @@
         <v>103</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="D81">
         <v>60</v>
@@ -5242,7 +5242,7 @@
         <v>105</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="D82">
         <v>100</v>
@@ -5270,7 +5270,7 @@
         <v>106</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="D83">
         <v>100</v>
@@ -5298,7 +5298,7 @@
         <v>107</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="D84">
         <v>55</v>
@@ -5326,7 +5326,7 @@
         <v>109</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="D85">
         <v>90</v>
@@ -5354,7 +5354,7 @@
         <v>110</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="D86">
         <v>130</v>
@@ -5382,7 +5382,7 @@
         <v>112</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="D87">
         <v>120</v>
@@ -5410,7 +5410,7 @@
         <v>113</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="D88">
         <v>120</v>
@@ -5438,7 +5438,7 @@
         <v>114</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="D89">
         <v>100</v>
@@ -5466,7 +5466,7 @@
         <v>115</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D90">
         <v>110</v>
@@ -5494,7 +5494,7 @@
         <v>116</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="D91">
         <v>140</v>
@@ -5522,7 +5522,7 @@
         <v>117</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="D92">
         <v>65</v>
@@ -5550,7 +5550,7 @@
         <v>118</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="D93">
         <v>40</v>
@@ -5578,7 +5578,7 @@
         <v>119</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="D94">
         <v>160</v>
@@ -5606,7 +5606,7 @@
         <v>120</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="D95">
         <v>130</v>
@@ -5634,7 +5634,7 @@
         <v>121</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="D96">
         <v>160</v>
@@ -5662,7 +5662,7 @@
         <v>123</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="D97">
         <v>120</v>
@@ -5690,7 +5690,7 @@
         <v>124</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="D98">
         <v>120</v>
@@ -5718,7 +5718,7 @@
         <v>125</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="D99">
         <v>120</v>
@@ -5746,7 +5746,7 @@
         <v>126</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="D100">
         <v>150</v>
@@ -5774,7 +5774,7 @@
         <v>127</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="D101">
         <v>90</v>
@@ -5802,7 +5802,7 @@
         <v>128</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="D102">
         <v>130</v>
@@ -5830,7 +5830,7 @@
         <v>130</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="D103">
         <v>60</v>
@@ -5858,7 +5858,7 @@
         <v>131</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D104">
         <v>60</v>
@@ -5886,7 +5886,7 @@
         <v>132</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="D105">
         <v>50</v>
@@ -5914,7 +5914,7 @@
         <v>133</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="D106">
         <v>60</v>
@@ -5942,7 +5942,7 @@
         <v>134</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="D107">
         <v>36</v>
@@ -5970,7 +5970,7 @@
         <v>135</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="D108">
         <v>50</v>
@@ -5998,7 +5998,7 @@
         <v>136</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D109">
         <v>45</v>
@@ -6026,7 +6026,7 @@
         <v>137</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="D110">
         <v>36</v>
@@ -6054,7 +6054,7 @@
         <v>138</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D111">
         <v>40</v>
@@ -6082,7 +6082,7 @@
         <v>140</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D112">
         <v>150</v>
@@ -6110,7 +6110,7 @@
         <v>141</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="D113">
         <v>150</v>
@@ -6138,7 +6138,7 @@
         <v>142</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="D114">
         <v>65</v>
@@ -6166,7 +6166,7 @@
         <v>143</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="D115">
         <v>60</v>
@@ -6194,7 +6194,7 @@
         <v>144</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="D116">
         <v>120</v>
@@ -6222,7 +6222,7 @@
         <v>146</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="D117">
         <v>38</v>
@@ -6250,7 +6250,7 @@
         <v>147</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D118">
         <v>55</v>
@@ -6278,7 +6278,7 @@
         <v>148</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="D119">
         <v>60</v>
@@ -6306,7 +6306,7 @@
         <v>149</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="D120">
         <v>60</v>
@@ -6334,7 +6334,7 @@
         <v>150</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="D121">
         <v>50</v>
@@ -6362,7 +6362,7 @@
         <v>151</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="D122">
         <v>60</v>
@@ -6390,7 +6390,7 @@
         <v>152</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="D123">
         <v>65</v>
@@ -6418,7 +6418,7 @@
         <v>153</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="D124">
         <v>60</v>
@@ -6446,7 +6446,7 @@
         <v>154</v>
       </c>
       <c r="C125" s="3" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="D125">
         <v>60</v>
@@ -6474,7 +6474,7 @@
         <v>156</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="D126">
         <v>100</v>
@@ -6502,7 +6502,7 @@
         <v>157</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="D127">
         <v>100</v>
@@ -6530,7 +6530,7 @@
         <v>158</v>
       </c>
       <c r="C128" s="3" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="D128">
         <v>90</v>
@@ -6558,7 +6558,7 @@
         <v>159</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="D129">
         <v>60</v>
@@ -6586,7 +6586,7 @@
         <v>160</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D130">
         <v>100</v>
@@ -6614,7 +6614,7 @@
         <v>161</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="D131">
         <v>55</v>
@@ -6642,7 +6642,7 @@
         <v>162</v>
       </c>
       <c r="C132" s="3" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="D132">
         <v>55</v>
@@ -6670,7 +6670,7 @@
         <v>163</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="D133">
         <v>90</v>
@@ -6698,7 +6698,7 @@
         <v>164</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="D134">
         <v>130</v>
@@ -6726,7 +6726,7 @@
         <v>165</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="D135">
         <v>120</v>
@@ -6754,7 +6754,7 @@
         <v>166</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="D136">
         <v>150</v>
@@ -6782,7 +6782,7 @@
         <v>167</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="D137">
         <v>100</v>
@@ -6810,7 +6810,7 @@
         <v>168</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="D138">
         <v>110</v>
@@ -6838,7 +6838,7 @@
         <v>169</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="D139">
         <v>110</v>
@@ -6866,7 +6866,7 @@
         <v>170</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="D140">
         <v>110</v>
@@ -6894,7 +6894,7 @@
         <v>171</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D141">
         <v>100</v>
@@ -6922,7 +6922,7 @@
         <v>172</v>
       </c>
       <c r="C142" s="3" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="D142">
         <v>50</v>
@@ -6950,7 +6950,7 @@
         <v>173</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D143">
         <v>50</v>
@@ -6978,7 +6978,7 @@
         <v>174</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D144">
         <v>55</v>
@@ -7006,7 +7006,7 @@
         <v>175</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D145">
         <v>50</v>
@@ -7034,7 +7034,7 @@
         <v>176</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D146">
         <v>50</v>
@@ -7062,7 +7062,7 @@
         <v>177</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="D147">
         <v>50</v>
@@ -7090,7 +7090,7 @@
         <v>178</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D148">
         <v>50</v>
@@ -7118,7 +7118,7 @@
         <v>179</v>
       </c>
       <c r="C149" s="3" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D149">
         <v>50</v>
@@ -7146,7 +7146,7 @@
         <v>181</v>
       </c>
       <c r="C150" s="3" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D150">
         <v>45</v>
@@ -7174,7 +7174,7 @@
         <v>182</v>
       </c>
       <c r="C151" s="3" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="D151">
         <v>50</v>
@@ -7202,7 +7202,7 @@
         <v>183</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D152">
         <v>40</v>
@@ -7230,7 +7230,7 @@
         <v>184</v>
       </c>
       <c r="C153" s="3" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="D153">
         <v>40</v>
@@ -7258,7 +7258,7 @@
         <v>185</v>
       </c>
       <c r="C154" s="3" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D154">
         <v>40</v>
@@ -7286,7 +7286,7 @@
         <v>186</v>
       </c>
       <c r="C155" s="3" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D155">
         <v>45</v>
@@ -7314,7 +7314,7 @@
         <v>187</v>
       </c>
       <c r="C156" s="3" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D156">
         <v>75</v>
@@ -7342,7 +7342,7 @@
         <v>188</v>
       </c>
       <c r="C157" s="3" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D157">
         <v>75</v>
@@ -7370,7 +7370,7 @@
         <v>189</v>
       </c>
       <c r="C158" s="3" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D158">
         <v>150</v>
@@ -7398,7 +7398,7 @@
         <v>190</v>
       </c>
       <c r="C159" s="3" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D159">
         <v>65</v>
@@ -7426,7 +7426,7 @@
         <v>191</v>
       </c>
       <c r="C160" s="3" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D160">
         <v>65</v>
@@ -7454,7 +7454,7 @@
         <v>192</v>
       </c>
       <c r="C161" s="3" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D161">
         <v>95</v>
@@ -7482,7 +7482,7 @@
         <v>193</v>
       </c>
       <c r="C162" s="3" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D162">
         <v>80</v>
@@ -7510,7 +7510,7 @@
         <v>194</v>
       </c>
       <c r="C163" s="3" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D163">
         <v>65</v>
@@ -7538,7 +7538,7 @@
         <v>195</v>
       </c>
       <c r="C164" s="3" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D164">
         <v>120</v>
@@ -7566,7 +7566,7 @@
         <v>196</v>
       </c>
       <c r="C165" s="3" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="D165">
         <v>80</v>
@@ -7594,7 +7594,7 @@
         <v>197</v>
       </c>
       <c r="C166" s="3" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="D166">
         <v>60</v>
@@ -7622,7 +7622,7 @@
         <v>198</v>
       </c>
       <c r="C167" s="3" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="D167">
         <v>140</v>
@@ -7650,7 +7650,7 @@
         <v>200</v>
       </c>
       <c r="C168" s="3" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D168">
         <v>80</v>
@@ -7678,7 +7678,7 @@
         <v>201</v>
       </c>
       <c r="C169" s="3" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="D169">
         <v>70</v>
@@ -7706,7 +7706,7 @@
         <v>202</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D170">
         <v>90</v>
@@ -7734,7 +7734,7 @@
         <v>203</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D171">
         <v>130</v>
@@ -7762,7 +7762,7 @@
         <v>205</v>
       </c>
       <c r="C172" s="3" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D172">
         <v>60</v>
@@ -7790,7 +7790,7 @@
         <v>206</v>
       </c>
       <c r="C173" s="3" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="D173">
         <v>60</v>
@@ -7818,7 +7818,7 @@
         <v>207</v>
       </c>
       <c r="C174" s="3" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D174">
         <v>60</v>
@@ -7846,7 +7846,7 @@
         <v>209</v>
       </c>
       <c r="C175" s="3" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D175">
         <v>50</v>
@@ -7874,7 +7874,7 @@
         <v>210</v>
       </c>
       <c r="C176" s="3" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D176">
         <v>50</v>
@@ -7902,7 +7902,7 @@
         <v>211</v>
       </c>
       <c r="C177" s="3" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D177">
         <v>60</v>
@@ -7930,7 +7930,7 @@
         <v>212</v>
       </c>
       <c r="C178" s="3" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D178">
         <v>60</v>
@@ -7958,7 +7958,7 @@
         <v>213</v>
       </c>
       <c r="C179" s="3" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="D179">
         <v>55</v>
@@ -7986,7 +7986,7 @@
         <v>214</v>
       </c>
       <c r="C180" s="3" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D180">
         <v>60</v>
@@ -8014,7 +8014,7 @@
         <v>216</v>
       </c>
       <c r="C181" s="3" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="D181">
         <v>140</v>
@@ -8042,7 +8042,7 @@
         <v>217</v>
       </c>
       <c r="C182" s="3" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D182">
         <v>80</v>
@@ -8070,7 +8070,7 @@
         <v>218</v>
       </c>
       <c r="C183" s="3" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="D183">
         <v>85</v>
@@ -8098,7 +8098,7 @@
         <v>219</v>
       </c>
       <c r="C184" s="3" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="D184">
         <v>60</v>
@@ -8126,7 +8126,7 @@
         <v>220</v>
       </c>
       <c r="C185" s="3" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="D185">
         <v>65</v>
@@ -8154,7 +8154,7 @@
         <v>222</v>
       </c>
       <c r="C186" s="3" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="D186">
         <v>140</v>
@@ -8182,7 +8182,7 @@
         <v>224</v>
       </c>
       <c r="C187" s="3" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="D187">
         <v>60</v>
@@ -8210,7 +8210,7 @@
         <v>226</v>
       </c>
       <c r="C188" s="3" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D188">
         <v>45</v>
@@ -8238,7 +8238,7 @@
         <v>228</v>
       </c>
       <c r="C189" s="3" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="D189">
         <v>65</v>
@@ -8266,7 +8266,7 @@
         <v>230</v>
       </c>
       <c r="C190" s="3" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D190">
         <v>80</v>
@@ -8294,7 +8294,7 @@
         <v>231</v>
       </c>
       <c r="C191" s="3" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="D191">
         <v>120</v>
@@ -8322,7 +8322,7 @@
         <v>233</v>
       </c>
       <c r="C192" s="3" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D192">
         <v>70</v>
@@ -8350,7 +8350,7 @@
         <v>234</v>
       </c>
       <c r="C193" s="3" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="D193">
         <v>80</v>
@@ -8378,7 +8378,7 @@
         <v>235</v>
       </c>
       <c r="C194" s="3" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="D194">
         <v>80</v>
@@ -8406,7 +8406,7 @@
         <v>237</v>
       </c>
       <c r="C195" s="3" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="D195">
         <v>80</v>
@@ -8434,7 +8434,7 @@
         <v>239</v>
       </c>
       <c r="C196" s="3" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D196">
         <v>160</v>
@@ -8462,7 +8462,7 @@
         <v>240</v>
       </c>
       <c r="C197" s="3" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="D197">
         <v>80</v>
@@ -8490,7 +8490,7 @@
         <v>241</v>
       </c>
       <c r="C198" s="3" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="D198">
         <v>120</v>
@@ -8518,7 +8518,7 @@
         <v>242</v>
       </c>
       <c r="C199" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="D199">
         <v>85</v>
@@ -8546,7 +8546,7 @@
         <v>243</v>
       </c>
       <c r="C200" s="3" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="D200">
         <v>85</v>
@@ -8574,7 +8574,7 @@
         <v>244</v>
       </c>
       <c r="C201" s="3" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="D201">
         <v>60</v>
@@ -8602,7 +8602,7 @@
         <v>245</v>
       </c>
       <c r="C202" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="D202">
         <v>60</v>
@@ -8630,7 +8630,7 @@
         <v>247</v>
       </c>
       <c r="C203" s="3" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="D203">
         <v>120</v>
@@ -8658,7 +8658,7 @@
         <v>249</v>
       </c>
       <c r="C204" s="3" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="D204">
         <v>130</v>
@@ -8686,7 +8686,7 @@
         <v>250</v>
       </c>
       <c r="C205" s="3" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="D205">
         <v>130</v>
@@ -8714,7 +8714,7 @@
         <v>251</v>
       </c>
       <c r="C206" s="3" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="D206">
         <v>130</v>
@@ -8742,7 +8742,7 @@
         <v>252</v>
       </c>
       <c r="C207" s="3" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="D207">
         <v>150</v>
@@ -8770,7 +8770,7 @@
         <v>253</v>
       </c>
       <c r="C208" s="3" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="D208">
         <v>65</v>
@@ -8798,7 +8798,7 @@
         <v>254</v>
       </c>
       <c r="C209" s="3" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="D209">
         <v>65</v>
@@ -8826,7 +8826,7 @@
         <v>255</v>
       </c>
       <c r="C210" s="3" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="D210">
         <v>65</v>
@@ -8854,7 +8854,7 @@
         <v>256</v>
       </c>
       <c r="C211" s="3" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="D211">
         <v>55</v>
@@ -8882,7 +8882,7 @@
         <v>257</v>
       </c>
       <c r="C212" s="3" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="D212">
         <v>65</v>
@@ -8910,7 +8910,7 @@
         <v>258</v>
       </c>
       <c r="C213" s="3" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="D213">
         <v>65</v>
@@ -8938,7 +8938,7 @@
         <v>259</v>
       </c>
       <c r="C214" s="3" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D214">
         <v>36</v>
@@ -8966,7 +8966,7 @@
         <v>261</v>
       </c>
       <c r="C215" s="3" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="D215">
         <v>130</v>
@@ -8994,7 +8994,7 @@
         <v>262</v>
       </c>
       <c r="C216" s="3" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D216">
         <v>120</v>
@@ -9022,7 +9022,7 @@
         <v>264</v>
       </c>
       <c r="C217" s="3" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="D217">
         <v>135</v>
@@ -9050,7 +9050,7 @@
         <v>265</v>
       </c>
       <c r="C218" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="D218">
         <v>140</v>
@@ -9078,7 +9078,7 @@
         <v>266</v>
       </c>
       <c r="C219" s="3" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="D219">
         <v>130</v>
@@ -9106,7 +9106,7 @@
         <v>267</v>
       </c>
       <c r="C220" s="3" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="D220">
         <v>130</v>
@@ -9134,7 +9134,7 @@
         <v>268</v>
       </c>
       <c r="C221" s="3" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="D221">
         <v>120</v>
@@ -9162,7 +9162,7 @@
         <v>269</v>
       </c>
       <c r="C222" s="3" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="D222">
         <v>25</v>
@@ -9190,7 +9190,7 @@
         <v>270</v>
       </c>
       <c r="C223" s="3" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="D223">
         <v>85</v>
@@ -9218,7 +9218,7 @@
         <v>271</v>
       </c>
       <c r="C224" s="3" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="D224">
         <v>85</v>
@@ -9246,7 +9246,7 @@
         <v>273</v>
       </c>
       <c r="C225" s="3" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="D225">
         <v>60</v>
@@ -9274,7 +9274,7 @@
         <v>275</v>
       </c>
       <c r="C226" s="3" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="D226">
         <v>80</v>
@@ -9302,7 +9302,7 @@
         <v>276</v>
       </c>
       <c r="C227" s="3" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="D227">
         <v>90</v>
@@ -9330,7 +9330,7 @@
         <v>277</v>
       </c>
       <c r="C228" s="3" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="D228">
         <v>90</v>
@@ -9358,7 +9358,7 @@
         <v>278</v>
       </c>
       <c r="C229" s="3" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="D229">
         <v>80</v>
@@ -9386,7 +9386,7 @@
         <v>280</v>
       </c>
       <c r="C230" s="3" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="D230">
         <v>105</v>
@@ -9414,7 +9414,7 @@
         <v>281</v>
       </c>
       <c r="C231" s="3" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="D231">
         <v>80</v>
@@ -9442,7 +9442,7 @@
         <v>283</v>
       </c>
       <c r="C232" s="3" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="D232">
         <v>90</v>
@@ -9470,7 +9470,7 @@
         <v>284</v>
       </c>
       <c r="C233" s="3" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="D233">
         <v>85</v>
@@ -9498,7 +9498,7 @@
         <v>286</v>
       </c>
       <c r="C234" s="3" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="D234">
         <v>100</v>
@@ -9526,7 +9526,7 @@
         <v>287</v>
       </c>
       <c r="C235" s="3" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="D235">
         <v>160</v>
@@ -9554,7 +9554,7 @@
         <v>289</v>
       </c>
       <c r="C236" s="3" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="D236">
         <v>110</v>
@@ -9582,7 +9582,7 @@
         <v>290</v>
       </c>
       <c r="C237" s="3" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="D237">
         <v>110</v>
@@ -9610,7 +9610,7 @@
         <v>291</v>
       </c>
       <c r="C238" s="3" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="D238">
         <v>120</v>
@@ -9638,7 +9638,7 @@
         <v>292</v>
       </c>
       <c r="C239" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="D239">
         <v>25</v>
@@ -9666,7 +9666,7 @@
         <v>293</v>
       </c>
       <c r="C240" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="D240">
         <v>160</v>
@@ -9694,7 +9694,7 @@
         <v>294</v>
       </c>
       <c r="C241" s="3" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="D241">
         <v>95</v>
@@ -9722,7 +9722,7 @@
         <v>295</v>
       </c>
       <c r="C242" s="3" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="D242">
         <v>80</v>
@@ -9750,7 +9750,7 @@
         <v>296</v>
       </c>
       <c r="C243" s="3" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="D243">
         <v>75</v>
@@ -9778,7 +9778,7 @@
         <v>297</v>
       </c>
       <c r="C244" s="3" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="D244">
         <v>45</v>
@@ -9806,7 +9806,7 @@
         <v>299</v>
       </c>
       <c r="C245" s="3" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="D245">
         <v>55</v>
@@ -9834,7 +9834,7 @@
         <v>301</v>
       </c>
       <c r="C246" s="3" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="D246">
         <v>50</v>
@@ -9862,7 +9862,7 @@
         <v>302</v>
       </c>
       <c r="C247" s="3" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="D247">
         <v>120</v>
@@ -9890,7 +9890,7 @@
         <v>303</v>
       </c>
       <c r="C248" s="3" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="D248">
         <v>110</v>
@@ -9918,7 +9918,7 @@
         <v>304</v>
       </c>
       <c r="C249" s="3" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="D249">
         <v>110</v>
@@ -9946,7 +9946,7 @@
         <v>305</v>
       </c>
       <c r="C250" s="3" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D250">
         <v>40</v>
@@ -9974,7 +9974,7 @@
         <v>307</v>
       </c>
       <c r="C251" s="3" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D251">
         <v>65</v>
@@ -10002,7 +10002,7 @@
         <v>308</v>
       </c>
       <c r="C252" s="3" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="D252">
         <v>50</v>
@@ -10030,7 +10030,7 @@
         <v>309</v>
       </c>
       <c r="C253" s="3" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="D253">
         <v>50</v>
@@ -10058,7 +10058,7 @@
         <v>310</v>
       </c>
       <c r="C254" s="3" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="D254">
         <v>55</v>
@@ -10086,7 +10086,7 @@
         <v>311</v>
       </c>
       <c r="C255" s="3" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="D255">
         <v>60</v>
@@ -10114,7 +10114,7 @@
         <v>313</v>
       </c>
       <c r="C256" s="3" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="D256">
         <v>85</v>
@@ -10142,7 +10142,7 @@
         <v>314</v>
       </c>
       <c r="C257" s="3" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="D257">
         <v>90</v>
@@ -10170,7 +10170,7 @@
         <v>315</v>
       </c>
       <c r="C258" s="3" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="D258">
         <v>30</v>
@@ -10198,7 +10198,7 @@
         <v>317</v>
       </c>
       <c r="C259" s="3" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="D259">
         <v>65</v>
@@ -10226,7 +10226,7 @@
         <v>319</v>
       </c>
       <c r="C260" s="3" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="D260">
         <v>45</v>
@@ -10254,7 +10254,7 @@
         <v>320</v>
       </c>
       <c r="C261" s="3" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="D261">
         <v>145</v>
@@ -10282,7 +10282,7 @@
         <v>321</v>
       </c>
       <c r="C262" s="3" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="D262">
         <v>140</v>
@@ -10310,7 +10310,7 @@
         <v>322</v>
       </c>
       <c r="C263" s="3" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D263">
         <v>140</v>
@@ -10338,7 +10338,7 @@
         <v>324</v>
       </c>
       <c r="C264" s="3" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="D264">
         <v>130</v>
@@ -10366,7 +10366,7 @@
         <v>326</v>
       </c>
       <c r="C265" s="3" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="D265">
         <v>130</v>
@@ -10394,7 +10394,7 @@
         <v>327</v>
       </c>
       <c r="C266" s="3" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="D266">
         <v>130</v>
@@ -10422,7 +10422,7 @@
         <v>328</v>
       </c>
       <c r="C267" s="3" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="D267">
         <v>130</v>
@@ -10450,7 +10450,7 @@
         <v>329</v>
       </c>
       <c r="C268" s="3" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="D268">
         <v>130</v>
@@ -10478,7 +10478,7 @@
         <v>330</v>
       </c>
       <c r="C269" s="3" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D269">
         <v>50</v>
@@ -10506,7 +10506,7 @@
         <v>331</v>
       </c>
       <c r="C270" s="3" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="D270">
         <v>110</v>
@@ -10534,7 +10534,7 @@
         <v>332</v>
       </c>
       <c r="C271" s="3" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="D271">
         <v>130</v>
@@ -10562,7 +10562,7 @@
         <v>333</v>
       </c>
       <c r="C272" s="3" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="D272">
         <v>100</v>
@@ -10590,7 +10590,7 @@
         <v>334</v>
       </c>
       <c r="C273" s="3" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="D273">
         <v>50</v>
@@ -10618,7 +10618,7 @@
         <v>335</v>
       </c>
       <c r="C274" s="3" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="D274">
         <v>50</v>
@@ -10646,7 +10646,7 @@
         <v>336</v>
       </c>
       <c r="C275" s="3" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="D275">
         <v>65</v>
@@ -10674,7 +10674,7 @@
         <v>337</v>
       </c>
       <c r="C276" s="3" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="D276">
         <v>140</v>
@@ -10702,7 +10702,7 @@
         <v>338</v>
       </c>
       <c r="C277" s="3" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="D277">
         <v>140</v>
@@ -10730,7 +10730,7 @@
         <v>339</v>
       </c>
       <c r="C278" s="3" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="D278">
         <v>160</v>
@@ -10758,7 +10758,7 @@
         <v>340</v>
       </c>
       <c r="C279" s="3" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="D279">
         <v>130</v>
@@ -10786,7 +10786,7 @@
         <v>341</v>
       </c>
       <c r="C280" s="3" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="D280">
         <v>130</v>
@@ -10814,7 +10814,7 @@
         <v>342</v>
       </c>
       <c r="C281" s="3" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="D281">
         <v>100</v>
@@ -10842,7 +10842,7 @@
         <v>343</v>
       </c>
       <c r="C282" s="3" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="D282">
         <v>55</v>
@@ -10870,7 +10870,7 @@
         <v>344</v>
       </c>
       <c r="C283" s="3" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="D283">
         <v>50</v>
@@ -10898,7 +10898,7 @@
         <v>345</v>
       </c>
       <c r="C284" s="3" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="D284">
         <v>55</v>
@@ -10926,7 +10926,7 @@
         <v>346</v>
       </c>
       <c r="C285" s="3" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="D285">
         <v>55</v>
@@ -10954,7 +10954,7 @@
         <v>347</v>
       </c>
       <c r="C286" s="3" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="D286">
         <v>85</v>
@@ -10982,7 +10982,7 @@
         <v>349</v>
       </c>
       <c r="C287" s="3" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="D287">
         <v>110</v>
@@ -11010,7 +11010,7 @@
         <v>350</v>
       </c>
       <c r="C288" s="3" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="D288">
         <v>110</v>
@@ -11038,7 +11038,7 @@
         <v>351</v>
       </c>
       <c r="C289" s="3" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="D289">
         <v>150</v>
@@ -11066,7 +11066,7 @@
         <v>352</v>
       </c>
       <c r="C290" s="3" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="D290">
         <v>110</v>
@@ -11094,7 +11094,7 @@
         <v>353</v>
       </c>
       <c r="C291" s="3" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="D291">
         <v>110</v>
@@ -11122,7 +11122,7 @@
         <v>354</v>
       </c>
       <c r="C292" s="3" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="D292">
         <v>85</v>
@@ -11150,7 +11150,7 @@
         <v>355</v>
       </c>
       <c r="C293" s="3" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="D293">
         <v>85</v>
@@ -11178,7 +11178,7 @@
         <v>356</v>
       </c>
       <c r="C294" s="3" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="D294">
         <v>140</v>
@@ -11206,7 +11206,7 @@
         <v>357</v>
       </c>
       <c r="C295" s="3" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="D295">
         <v>130</v>
@@ -11234,7 +11234,7 @@
         <v>358</v>
       </c>
       <c r="C296" s="3" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="D296">
         <v>150</v>
@@ -11262,7 +11262,7 @@
         <v>359</v>
       </c>
       <c r="C297" s="3" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="D297">
         <v>135</v>
@@ -11290,7 +11290,7 @@
         <v>360</v>
       </c>
       <c r="C298" s="3" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="D298">
         <v>150</v>
@@ -11318,7 +11318,7 @@
         <v>361</v>
       </c>
       <c r="C299" s="3" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D299">
         <v>65</v>
@@ -11346,7 +11346,7 @@
         <v>362</v>
       </c>
       <c r="C300" s="3" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="D300">
         <v>90</v>
@@ -11374,7 +11374,7 @@
         <v>363</v>
       </c>
       <c r="C301" s="3" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="D301">
         <v>90</v>
@@ -11402,7 +11402,7 @@
         <v>364</v>
       </c>
       <c r="C302" s="3" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="D302">
         <v>90</v>
@@ -11430,7 +11430,7 @@
         <v>365</v>
       </c>
       <c r="C303" s="3" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="D303">
         <v>90</v>
@@ -11458,7 +11458,7 @@
         <v>366</v>
       </c>
       <c r="C304" s="3" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="D304">
         <v>90</v>
@@ -11486,7 +11486,7 @@
         <v>367</v>
       </c>
       <c r="C305" s="3" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="D305">
         <v>90</v>
@@ -11514,7 +11514,7 @@
         <v>368</v>
       </c>
       <c r="C306" s="3" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="D306">
         <v>120</v>
@@ -11542,7 +11542,7 @@
         <v>370</v>
       </c>
       <c r="C307" s="3" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="D307">
         <v>70</v>
@@ -11570,7 +11570,7 @@
         <v>371</v>
       </c>
       <c r="C308" s="3" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="D308">
         <v>150</v>
@@ -11598,7 +11598,7 @@
         <v>373</v>
       </c>
       <c r="C309" s="3" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="D309">
         <v>110</v>
@@ -11626,7 +11626,7 @@
         <v>374</v>
       </c>
       <c r="C310" s="3" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="D310">
         <v>90</v>
@@ -11654,7 +11654,7 @@
         <v>375</v>
       </c>
       <c r="C311" s="3" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="D311">
         <v>90</v>
@@ -11682,7 +11682,7 @@
         <v>376</v>
       </c>
       <c r="C312" s="3" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="D312">
         <v>85</v>
@@ -11710,7 +11710,7 @@
         <v>377</v>
       </c>
       <c r="C313" s="3" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="D313">
         <v>90</v>
@@ -11738,7 +11738,7 @@
         <v>379</v>
       </c>
       <c r="C314" s="3" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="D314">
         <v>90</v>
@@ -11766,7 +11766,7 @@
         <v>380</v>
       </c>
       <c r="C315" s="3" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="D315">
         <v>90</v>
@@ -11794,7 +11794,7 @@
         <v>381</v>
       </c>
       <c r="C316" s="3" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="D316">
         <v>150</v>
@@ -11822,7 +11822,7 @@
         <v>382</v>
       </c>
       <c r="C317" s="3" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="D317">
         <v>160</v>
@@ -11850,7 +11850,7 @@
         <v>383</v>
       </c>
       <c r="C318" s="3" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="D318">
         <v>160</v>
@@ -11878,7 +11878,7 @@
         <v>384</v>
       </c>
       <c r="C319" s="3" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="D319">
         <v>140</v>
@@ -11906,7 +11906,7 @@
         <v>385</v>
       </c>
       <c r="C320" s="3" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="D320">
         <v>135</v>
@@ -11934,7 +11934,7 @@
         <v>386</v>
       </c>
       <c r="C321" s="3" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="D321">
         <v>135</v>
@@ -11962,7 +11962,7 @@
         <v>387</v>
       </c>
       <c r="C322" s="3" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D322">
         <v>140</v>
@@ -11990,7 +11990,7 @@
         <v>388</v>
       </c>
       <c r="C323" s="3" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="D323">
         <v>120</v>
@@ -12018,7 +12018,7 @@
         <v>389</v>
       </c>
       <c r="C324" s="3" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="D324">
         <v>140</v>
@@ -12046,7 +12046,7 @@
         <v>390</v>
       </c>
       <c r="C325" s="3" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="D325">
         <v>120</v>
@@ -12074,7 +12074,7 @@
         <v>391</v>
       </c>
       <c r="C326" s="3" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="D326">
         <v>120</v>
@@ -12102,7 +12102,7 @@
         <v>392</v>
       </c>
       <c r="C327" s="3" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="D327">
         <v>140</v>
@@ -12130,7 +12130,7 @@
         <v>393</v>
       </c>
       <c r="C328" s="3" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="D328">
         <v>100</v>
@@ -12158,7 +12158,7 @@
         <v>394</v>
       </c>
       <c r="C329" s="3" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="D329">
         <v>85</v>
@@ -12186,7 +12186,7 @@
         <v>396</v>
       </c>
       <c r="C330" s="3" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="D330">
         <v>50</v>
@@ -12214,7 +12214,7 @@
         <v>397</v>
       </c>
       <c r="C331" s="3" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="D331">
         <v>50</v>
@@ -12242,7 +12242,7 @@
         <v>398</v>
       </c>
       <c r="C332" s="3" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="D332">
         <v>50</v>
@@ -12270,7 +12270,7 @@
         <v>400</v>
       </c>
       <c r="C333" s="3" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="D333">
         <v>45</v>
@@ -12298,7 +12298,7 @@
         <v>401</v>
       </c>
       <c r="C334" s="3" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="D334">
         <v>90</v>
@@ -12326,7 +12326,7 @@
         <v>403</v>
       </c>
       <c r="C335" s="3" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="D335">
         <v>85</v>
@@ -12354,7 +12354,7 @@
         <v>405</v>
       </c>
       <c r="C336" s="3" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="D336">
         <v>70</v>
@@ -12382,7 +12382,7 @@
         <v>407</v>
       </c>
       <c r="C337" s="3" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="D337">
         <v>60</v>
@@ -12410,7 +12410,7 @@
         <v>408</v>
       </c>
       <c r="C338" s="3" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="D338">
         <v>90</v>
@@ -12438,7 +12438,7 @@
         <v>409</v>
       </c>
       <c r="C339" s="3" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="D339">
         <v>130</v>
@@ -12466,7 +12466,7 @@
         <v>411</v>
       </c>
       <c r="C340" s="3" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="D340">
         <v>150</v>
@@ -12494,7 +12494,7 @@
         <v>413</v>
       </c>
       <c r="C341" s="3" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="D341">
         <v>120</v>
@@ -12522,7 +12522,7 @@
         <v>415</v>
       </c>
       <c r="C342" s="3" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="D342">
         <v>140</v>
@@ -12550,7 +12550,7 @@
         <v>416</v>
       </c>
       <c r="C343" s="3" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="D343">
         <v>135</v>
@@ -12578,7 +12578,7 @@
         <v>417</v>
       </c>
       <c r="C344" s="3" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="D344">
         <v>135</v>
@@ -12606,7 +12606,7 @@
         <v>418</v>
       </c>
       <c r="C345" s="3" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="D345">
         <v>160</v>
@@ -12634,7 +12634,7 @@
         <v>419</v>
       </c>
       <c r="C346" s="3" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="D346">
         <v>140</v>
@@ -12662,7 +12662,7 @@
         <v>420</v>
       </c>
       <c r="C347" s="3" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D347">
         <v>160</v>
@@ -12690,7 +12690,7 @@
         <v>421</v>
       </c>
       <c r="C348" s="3" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D348">
         <v>140</v>
@@ -12718,7 +12718,7 @@
         <v>422</v>
       </c>
       <c r="C349" s="3" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="D349">
         <v>150</v>
@@ -12746,7 +12746,7 @@
         <v>423</v>
       </c>
       <c r="C350" s="3" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="D350">
         <v>150</v>
@@ -12774,7 +12774,7 @@
         <v>424</v>
       </c>
       <c r="C351" s="3" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="D351">
         <v>140</v>
@@ -12802,7 +12802,7 @@
         <v>425</v>
       </c>
       <c r="C352" s="3" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="D352">
         <v>85</v>
@@ -12830,7 +12830,7 @@
         <v>426</v>
       </c>
       <c r="C353" s="3" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="D353">
         <v>90</v>
@@ -12858,7 +12858,7 @@
         <v>427</v>
       </c>
       <c r="C354" s="3" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="D354">
         <v>90</v>
@@ -12886,7 +12886,7 @@
         <v>429</v>
       </c>
       <c r="C355" s="3" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D355">
         <v>65</v>
@@ -12914,7 +12914,7 @@
         <v>430</v>
       </c>
       <c r="C356" s="3" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="D356">
         <v>35</v>
@@ -12942,7 +12942,7 @@
         <v>431</v>
       </c>
       <c r="C357" s="3" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="D357">
         <v>90</v>
@@ -12970,7 +12970,7 @@
         <v>432</v>
       </c>
       <c r="C358" s="3" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="D358">
         <v>85</v>
@@ -12998,7 +12998,7 @@
         <v>433</v>
       </c>
       <c r="C359" s="3" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D359">
         <v>85</v>
@@ -13026,7 +13026,7 @@
         <v>434</v>
       </c>
       <c r="C360" s="3" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="D360">
         <v>85</v>
@@ -13054,7 +13054,7 @@
         <v>435</v>
       </c>
       <c r="C361" s="3" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="D361">
         <v>85</v>
@@ -13082,7 +13082,7 @@
         <v>436</v>
       </c>
       <c r="C362" s="3" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="D362">
         <v>90</v>
@@ -13110,7 +13110,7 @@
         <v>437</v>
       </c>
       <c r="C363" s="3" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="D363">
         <v>60</v>
@@ -13138,7 +13138,7 @@
         <v>438</v>
       </c>
       <c r="C364" s="3" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="D364">
         <v>70</v>
@@ -13166,7 +13166,7 @@
         <v>439</v>
       </c>
       <c r="C365" s="3" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="D365">
         <v>70</v>
@@ -13194,7 +13194,7 @@
         <v>440</v>
       </c>
       <c r="C366" s="3" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="D366">
         <v>65</v>
@@ -13222,7 +13222,7 @@
         <v>441</v>
       </c>
       <c r="C367" s="3" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="D367">
         <v>60</v>
@@ -13250,7 +13250,7 @@
         <v>442</v>
       </c>
       <c r="C368" s="3" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D368">
         <v>65</v>
@@ -13278,7 +13278,7 @@
         <v>443</v>
       </c>
       <c r="C369" s="3" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D369">
         <v>65</v>
@@ -13306,7 +13306,7 @@
         <v>444</v>
       </c>
       <c r="C370" s="3" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="D370">
         <v>65</v>
@@ -13334,7 +13334,7 @@
         <v>445</v>
       </c>
       <c r="C371" s="3" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="D371">
         <v>90</v>
@@ -13362,7 +13362,7 @@
         <v>446</v>
       </c>
       <c r="C372" s="3" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="D372">
         <v>36</v>
@@ -13390,7 +13390,7 @@
         <v>447</v>
       </c>
       <c r="C373" s="3" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="D373">
         <v>85</v>
@@ -13418,7 +13418,7 @@
         <v>448</v>
       </c>
       <c r="C374" s="3" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D374">
         <v>130</v>
@@ -13446,7 +13446,7 @@
         <v>449</v>
       </c>
       <c r="C375" s="3" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="D375">
         <v>60</v>
@@ -13474,7 +13474,7 @@
         <v>450</v>
       </c>
       <c r="C376" s="3" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D376">
         <v>60</v>
@@ -13502,7 +13502,7 @@
         <v>451</v>
       </c>
       <c r="C377" s="3" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="D377">
         <v>65</v>
@@ -13530,7 +13530,7 @@
         <v>452</v>
       </c>
       <c r="C378" s="3" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="D378">
         <v>55</v>
@@ -13558,7 +13558,7 @@
         <v>453</v>
       </c>
       <c r="C379" s="3" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="D379">
         <v>55</v>
@@ -13586,7 +13586,7 @@
         <v>454</v>
       </c>
       <c r="C380" s="3" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="D380">
         <v>60</v>
@@ -13614,7 +13614,7 @@
         <v>455</v>
       </c>
       <c r="C381" s="3" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="D381">
         <v>65</v>
@@ -13642,7 +13642,7 @@
         <v>457</v>
       </c>
       <c r="C382" s="3" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="D382">
         <v>70</v>
@@ -13670,7 +13670,7 @@
         <v>458</v>
       </c>
       <c r="C383" s="3" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D383">
         <v>55</v>
@@ -13698,7 +13698,7 @@
         <v>459</v>
       </c>
       <c r="C384" s="3" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="D384">
         <v>140</v>

</xml_diff>